<commit_message>
refactor: restructure validation logic inside try blovk and Validate TC07 happy path
</commit_message>
<xml_diff>
--- a/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
+++ b/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
@@ -4,15 +4,16 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="TC01" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="TC02" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="TC03" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="TC04" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="TC05" sheetId="5" r:id="rId9"/>
-    <sheet state="visible" name="TC06" sheetId="6" r:id="rId10"/>
-    <sheet state="visible" name="TC07" sheetId="7" r:id="rId11"/>
-    <sheet state="visible" name="TC08" sheetId="8" r:id="rId12"/>
-    <sheet state="visible" name="Hoja 12" sheetId="9" r:id="rId13"/>
-    <sheet state="visible" name="TC Codigo" sheetId="10" r:id="rId14"/>
+    <sheet state="visible" name="EX1" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="TC02" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="TC03" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="TC04" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="TC05" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="TC06" sheetId="7" r:id="rId11"/>
+    <sheet state="visible" name="TC07" sheetId="8" r:id="rId12"/>
+    <sheet state="visible" name="TC08" sheetId="9" r:id="rId13"/>
+    <sheet state="visible" name="Hoja 12" sheetId="10" r:id="rId14"/>
+    <sheet state="visible" name="TC Codigo" sheetId="11" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="118">
   <si>
     <t>date</t>
   </si>
@@ -220,6 +221,9 @@
     <t>Review</t>
   </si>
   <si>
+    <t>Observaciones de test</t>
+  </si>
+  <si>
     <t>Excepción por Archivo Inexistente</t>
   </si>
   <si>
@@ -244,6 +248,9 @@
     <t xml:space="preserve">en el script el usuario escribe ReporteMayo y es reportemayo </t>
   </si>
   <si>
+    <t>Pending</t>
+  </si>
+  <si>
     <t>Invalidez de Metadatos de Pestaña</t>
   </si>
   <si>
@@ -277,10 +284,16 @@
     <t>La columa de informacion requerida no existe, es decir, fecha, campaña, comienza directo con los datos crudo fechas, camapañas, numeros sind escripcion o bien puede faltar solo 1 datos e indicar que datos faltan</t>
   </si>
   <si>
+    <t>El programa indice cuando Falta solo una columa, e infdica el nombre, si faltan mas indica las que falten, si faltan todasde igual forma lo dice esto cuando analiza desde la A1 a lo que sigue</t>
+  </si>
+  <si>
     <t>Caso Feliz (Estructura Óptima)</t>
   </si>
   <si>
     <t>Óptima)El archivo se presenta con el esquema, orden y tipos de datos correctos. Se procesa sin registrar alertas.</t>
+  </si>
+  <si>
+    <t>Se sube el archivo de prueba en la hoja debira con datos completos y sevisualiza que al finalizar el programa analiza las columnase indica  que estan completos los datos</t>
   </si>
   <si>
     <t>Desfase de Origen Vertical (Filas basura al inicio</t>
@@ -371,7 +384,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/M/yyyy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -387,8 +400,13 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -407,14 +425,57 @@
         <bgColor rgb="FF4DD0E1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6AA84F"/>
+        <bgColor rgb="FF6AA84F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1C232"/>
+        <bgColor rgb="FFF1C232"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFCC0000"/>
+        <bgColor rgb="FFCC0000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="36">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -454,7 +515,19 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -463,26 +536,53 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -562,6 +662,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
@@ -599,14 +703,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F24" displayName="Tabla_1" name="Tabla_1" id="1">
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:G24" displayName="Tabla_1" name="Tabla_1" id="1">
+  <tableColumns count="7">
     <tableColumn name="Case" id="1"/>
     <tableColumn name="Defecto a revisar" id="2"/>
     <tableColumn name="Descripcion" id="3"/>
     <tableColumn name="Notas" id="4"/>
     <tableColumn name="Status" id="5"/>
     <tableColumn name="Review" id="6"/>
+    <tableColumn name="Observaciones de test" id="7"/>
   </tableColumns>
   <tableStyleInfo name="TC Codigo-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
@@ -1222,11 +1327,426 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="47.38"/>
-    <col customWidth="1" min="3" max="3" width="46.13"/>
+    <col customWidth="1" min="1" max="1" width="18.38"/>
+    <col customWidth="1" min="2" max="2" width="18.0"/>
+    <col customWidth="1" min="3" max="3" width="14.88"/>
+    <col customWidth="1" min="4" max="4" width="18.25"/>
+    <col customWidth="1" min="5" max="5" width="80.5"/>
+    <col customWidth="1" min="6" max="6" width="15.13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="28.63"/>
+    <col customWidth="1" min="3" max="3" width="41.75"/>
     <col customWidth="1" min="4" max="4" width="33.75"/>
     <col customWidth="1" min="5" max="5" width="25.75"/>
     <col customWidth="1" min="6" max="6" width="22.63"/>
+    <col customWidth="1" min="7" max="7" width="23.75"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
@@ -1248,7 +1768,9 @@
       <c r="F1" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="G1" s="12"/>
+      <c r="G1" s="11" t="s">
+        <v>66</v>
+      </c>
       <c r="H1" s="12"/>
       <c r="I1" s="12"/>
     </row>
@@ -1256,389 +1778,410 @@
       <c r="A2" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="C2" s="14" t="s">
+      <c r="B2" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="C2" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="D2" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="E2" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="G2" s="12"/>
+      <c r="F2" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="G2" s="14"/>
       <c r="H2" s="12"/>
       <c r="I2" s="12"/>
     </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="C3" s="14" t="s">
+      <c r="B3" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="C3" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="14"/>
+      <c r="D3" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="F3" s="16"/>
-      <c r="G3" s="12"/>
+      <c r="G3" s="16"/>
       <c r="H3" s="12"/>
       <c r="I3" s="12"/>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="C4" s="14" t="s">
+      <c r="B4" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="E4" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="D4" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="E4" s="14"/>
       <c r="F4" s="16"/>
-      <c r="G4" s="12"/>
+      <c r="G4" s="16"/>
       <c r="H4" s="12"/>
       <c r="I4" s="12"/>
     </row>
     <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="D5" s="14" t="s">
+      <c r="B5" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="E5" s="14"/>
+      <c r="C5" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="F5" s="16"/>
-      <c r="G5" s="12"/>
+      <c r="G5" s="16"/>
       <c r="H5" s="12"/>
       <c r="I5" s="12"/>
     </row>
     <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" s="14" t="s">
+      <c r="B6" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="E6" s="14"/>
+      <c r="C6" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="F6" s="16"/>
-      <c r="G6" s="12"/>
+      <c r="G6" s="17"/>
       <c r="H6" s="12"/>
       <c r="I6" s="12"/>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="14"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="12"/>
+      <c r="A7" s="18"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
       <c r="H7" s="12"/>
       <c r="I7" s="12"/>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="14"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="12"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
       <c r="H8" s="12"/>
       <c r="I8" s="12"/>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="C9" s="14" t="s">
+      <c r="B9" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="14"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="12"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
       <c r="H9" s="12"/>
       <c r="I9" s="12"/>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="D10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="E10" s="14"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="12"/>
+      <c r="C10" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13" t="s">
+        <v>87</v>
+      </c>
       <c r="H10" s="12"/>
       <c r="I10" s="12"/>
     </row>
     <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B11" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="D11" s="18"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="12"/>
+      <c r="B11" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="D11" s="22"/>
+      <c r="E11" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" s="14"/>
+      <c r="G11" s="13" t="s">
+        <v>90</v>
+      </c>
       <c r="H11" s="12"/>
       <c r="I11" s="12"/>
     </row>
     <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="E12" s="14"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="12"/>
+      <c r="B12" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="E12" s="23"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
     </row>
     <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="E13" s="14"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="12"/>
+      <c r="B13" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="E13" s="23"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
     </row>
     <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="E14" s="14"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="12"/>
+      <c r="B14" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="E14" s="23"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
       <c r="H14" s="12"/>
       <c r="I14" s="12"/>
     </row>
     <row r="15" ht="22.5" customHeight="1">
-      <c r="A15" s="18"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="12"/>
+      <c r="A15" s="25"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
       <c r="H15" s="12"/>
       <c r="I15" s="12"/>
     </row>
     <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="18"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="12"/>
+      <c r="A16" s="25"/>
+      <c r="B16" s="25"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
     </row>
     <row r="17" ht="22.5" customHeight="1">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="C17" s="14" t="s">
+      <c r="B17" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="D17" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="E17" s="18"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="12"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
     </row>
     <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="E18" s="18"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="12"/>
+      <c r="B18" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>101</v>
+      </c>
+      <c r="D18" s="28" t="s">
+        <v>102</v>
+      </c>
+      <c r="E18" s="29"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
     </row>
     <row r="19" ht="22.5" customHeight="1">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="D19" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="E19" s="18"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="12"/>
+      <c r="B19" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="E19" s="29"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
     </row>
     <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="E20" s="18"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="12"/>
+      <c r="B20" s="28" t="s">
+        <v>106</v>
+      </c>
+      <c r="C20" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="D20" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="E20" s="29"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
       <c r="H20" s="12"/>
       <c r="I20" s="12"/>
     </row>
     <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="B21" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="E21" s="18"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="12"/>
+      <c r="B21" s="28" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="D21" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="E21" s="29"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="30"/>
       <c r="H21" s="12"/>
       <c r="I21" s="12"/>
     </row>
     <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="31" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="21" t="s">
-        <v>108</v>
-      </c>
-      <c r="C22" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="F22" s="22"/>
+      <c r="B22" s="32" t="s">
+        <v>112</v>
+      </c>
+      <c r="C22" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="D22" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="E22" s="33"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
     </row>
     <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="F23" s="22"/>
+      <c r="B23" s="32" t="s">
+        <v>115</v>
+      </c>
+      <c r="C23" s="32" t="s">
+        <v>116</v>
+      </c>
+      <c r="D23" s="28" t="s">
+        <v>117</v>
+      </c>
+      <c r="E23" s="33"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="34"/>
     </row>
     <row r="24" ht="22.5" customHeight="1">
-      <c r="A24" s="18"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="19"/>
+      <c r="A24" s="25"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="35"/>
+      <c r="G24" s="35"/>
     </row>
     <row r="26">
       <c r="C26" s="7"/>
@@ -1661,30 +2204,160 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
+    <row r="1">
+      <c r="A1" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="5">
+        <v>5168.0</v>
+      </c>
+      <c r="E1" s="5">
+        <v>134.0</v>
+      </c>
+      <c r="F1" s="5">
+        <v>258.0</v>
+      </c>
+      <c r="G1" s="4">
+        <v>362.0</v>
+      </c>
+      <c r="H1" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="5">
+        <v>2314.0</v>
+      </c>
+      <c r="E2" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="F2" s="5">
+        <v>162.0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>46.0</v>
+      </c>
+      <c r="H2" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5">
+        <v>3496.0</v>
+      </c>
+      <c r="E3" s="5">
+        <v>92.0</v>
+      </c>
+      <c r="F3" s="5">
+        <v>61.0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="H3" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1790.0</v>
+      </c>
+      <c r="E4" s="5">
+        <v>87.0</v>
+      </c>
+      <c r="F4" s="5">
+        <v>370.0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>54.0</v>
+      </c>
+      <c r="H4" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="5">
+        <v>9764.0</v>
+      </c>
+      <c r="E5" s="5">
+        <v>53.0</v>
+      </c>
+      <c r="F5" s="5">
+        <v>118.0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>293.0</v>
+      </c>
+      <c r="H5" s="6">
+        <v>3.0</v>
+      </c>
+    </row>
     <row r="6">
-      <c r="A6" s="1" t="s">
-        <v>0</v>
+      <c r="A6" s="4">
+        <v>45658.0</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>7</v>
+        <v>14</v>
+      </c>
+      <c r="D6" s="5">
+        <v>2912.0</v>
+      </c>
+      <c r="E6" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="F6" s="5">
+        <v>187.0</v>
+      </c>
+      <c r="G6" s="4">
+        <v>204.0</v>
+      </c>
+      <c r="H6" s="6">
+        <v>1.0</v>
       </c>
     </row>
     <row r="7">
@@ -1695,22 +2368,22 @@
         <v>8</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D7" s="5">
-        <v>5168.0</v>
+        <v>4736.0</v>
       </c>
       <c r="E7" s="5">
-        <v>134.0</v>
+        <v>123.0</v>
       </c>
       <c r="F7" s="5">
-        <v>258.0</v>
+        <v>198.0</v>
       </c>
       <c r="G7" s="4">
-        <v>362.0</v>
+        <v>237.0</v>
       </c>
       <c r="H7" s="6">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="8">
@@ -1718,25 +2391,25 @@
         <v>45658.0</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8" s="5">
-        <v>2314.0</v>
+        <v>7311.0</v>
       </c>
       <c r="E8" s="5">
-        <v>26.0</v>
+        <v>149.0</v>
       </c>
       <c r="F8" s="5">
-        <v>162.0</v>
+        <v>230.0</v>
       </c>
       <c r="G8" s="4">
-        <v>46.0</v>
+        <v>219.0</v>
       </c>
       <c r="H8" s="6">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="9">
@@ -1744,22 +2417,22 @@
         <v>45658.0</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" s="5">
-        <v>3496.0</v>
+        <v>4679.0</v>
       </c>
       <c r="E9" s="5">
-        <v>92.0</v>
+        <v>22.0</v>
       </c>
       <c r="F9" s="5">
-        <v>61.0</v>
+        <v>281.0</v>
       </c>
       <c r="G9" s="4">
-        <v>175.0</v>
+        <v>94.0</v>
       </c>
       <c r="H9" s="6">
         <v>1.0</v>
@@ -1770,25 +2443,25 @@
         <v>45658.0</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D10" s="5">
-        <v>1790.0</v>
+        <v>4957.0</v>
       </c>
       <c r="E10" s="5">
-        <v>87.0</v>
+        <v>93.0</v>
       </c>
       <c r="F10" s="5">
-        <v>370.0</v>
+        <v>276.0</v>
       </c>
       <c r="G10" s="4">
-        <v>54.0</v>
+        <v>397.0</v>
       </c>
       <c r="H10" s="6">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="11">
@@ -1796,258 +2469,102 @@
         <v>45658.0</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D11" s="5">
-        <v>9764.0</v>
+        <v>2924.0</v>
       </c>
       <c r="E11" s="5">
-        <v>53.0</v>
+        <v>131.0</v>
       </c>
       <c r="F11" s="5">
-        <v>118.0</v>
+        <v>58.0</v>
       </c>
       <c r="G11" s="4">
-        <v>293.0</v>
+        <v>175.0</v>
       </c>
       <c r="H11" s="6">
-        <v>3.0</v>
+        <v>7.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4">
         <v>45658.0</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>14</v>
+      <c r="B12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>13</v>
       </c>
       <c r="D12" s="5">
-        <v>2912.0</v>
+        <v>7200.0</v>
       </c>
       <c r="E12" s="5">
-        <v>26.0</v>
+        <v>96.0</v>
       </c>
       <c r="F12" s="5">
-        <v>187.0</v>
-      </c>
-      <c r="G12" s="4">
-        <v>204.0</v>
+        <v>315.0</v>
+      </c>
+      <c r="G12" s="6">
+        <v>288.0</v>
       </c>
       <c r="H12" s="6">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4">
         <v>45658.0</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>15</v>
+      <c r="B13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="D13" s="5">
-        <v>4736.0</v>
+        <v>2177.0</v>
       </c>
       <c r="E13" s="5">
-        <v>123.0</v>
+        <v>23.0</v>
       </c>
       <c r="F13" s="5">
-        <v>198.0</v>
-      </c>
-      <c r="G13" s="4">
-        <v>237.0</v>
+        <v>262.0</v>
+      </c>
+      <c r="G13" s="6">
+        <v>131.0</v>
       </c>
       <c r="H13" s="6">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4">
         <v>45658.0</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>9</v>
+      <c r="B14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="D14" s="5">
-        <v>7311.0</v>
+        <v>4367.0</v>
       </c>
       <c r="E14" s="5">
-        <v>149.0</v>
+        <v>126.0</v>
       </c>
       <c r="F14" s="5">
-        <v>230.0</v>
-      </c>
-      <c r="G14" s="4">
-        <v>219.0</v>
+        <v>161.0</v>
+      </c>
+      <c r="G14" s="6">
+        <v>262.0</v>
       </c>
       <c r="H14" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="5">
-        <v>4679.0</v>
-      </c>
-      <c r="E15" s="5">
-        <v>22.0</v>
-      </c>
-      <c r="F15" s="5">
-        <v>281.0</v>
-      </c>
-      <c r="G15" s="4">
-        <v>94.0</v>
-      </c>
-      <c r="H15" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="5">
-        <v>4957.0</v>
-      </c>
-      <c r="E16" s="5">
-        <v>93.0</v>
-      </c>
-      <c r="F16" s="5">
-        <v>276.0</v>
-      </c>
-      <c r="G16" s="4">
-        <v>397.0</v>
-      </c>
-      <c r="H16" s="6">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="5">
-        <v>2924.0</v>
-      </c>
-      <c r="E17" s="5">
-        <v>131.0</v>
-      </c>
-      <c r="F17" s="5">
-        <v>58.0</v>
-      </c>
-      <c r="G17" s="4">
-        <v>175.0</v>
-      </c>
-      <c r="H17" s="6">
-        <v>7.0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" s="5">
-        <v>7200.0</v>
-      </c>
-      <c r="E18" s="5">
-        <v>96.0</v>
-      </c>
-      <c r="F18" s="5">
-        <v>315.0</v>
-      </c>
-      <c r="G18" s="6">
-        <v>288.0</v>
-      </c>
-      <c r="H18" s="6">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19" s="5">
-        <v>2177.0</v>
-      </c>
-      <c r="E19" s="5">
-        <v>23.0</v>
-      </c>
-      <c r="F19" s="5">
-        <v>262.0</v>
-      </c>
-      <c r="G19" s="6">
-        <v>131.0</v>
-      </c>
-      <c r="H19" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D20" s="5">
-        <v>4367.0</v>
-      </c>
-      <c r="E20" s="5">
-        <v>126.0</v>
-      </c>
-      <c r="F20" s="5">
-        <v>161.0</v>
-      </c>
-      <c r="G20" s="6">
-        <v>262.0</v>
-      </c>
-      <c r="H20" s="6">
         <v>6.0</v>
       </c>
     </row>
@@ -2057,6 +2574,408 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="6">
+      <c r="A6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="5">
+        <v>5168.0</v>
+      </c>
+      <c r="E7" s="5">
+        <v>134.0</v>
+      </c>
+      <c r="F7" s="5">
+        <v>258.0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>362.0</v>
+      </c>
+      <c r="H7" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="5">
+        <v>2314.0</v>
+      </c>
+      <c r="E8" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="F8" s="5">
+        <v>162.0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>46.0</v>
+      </c>
+      <c r="H8" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="5">
+        <v>3496.0</v>
+      </c>
+      <c r="E9" s="5">
+        <v>92.0</v>
+      </c>
+      <c r="F9" s="5">
+        <v>61.0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="H9" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="5">
+        <v>1790.0</v>
+      </c>
+      <c r="E10" s="5">
+        <v>87.0</v>
+      </c>
+      <c r="F10" s="5">
+        <v>370.0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>54.0</v>
+      </c>
+      <c r="H10" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="5">
+        <v>9764.0</v>
+      </c>
+      <c r="E11" s="5">
+        <v>53.0</v>
+      </c>
+      <c r="F11" s="5">
+        <v>118.0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>293.0</v>
+      </c>
+      <c r="H11" s="6">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="5">
+        <v>2912.0</v>
+      </c>
+      <c r="E12" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="F12" s="5">
+        <v>187.0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>204.0</v>
+      </c>
+      <c r="H12" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="5">
+        <v>4736.0</v>
+      </c>
+      <c r="E13" s="5">
+        <v>123.0</v>
+      </c>
+      <c r="F13" s="5">
+        <v>198.0</v>
+      </c>
+      <c r="G13" s="4">
+        <v>237.0</v>
+      </c>
+      <c r="H13" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="5">
+        <v>7311.0</v>
+      </c>
+      <c r="E14" s="5">
+        <v>149.0</v>
+      </c>
+      <c r="F14" s="5">
+        <v>230.0</v>
+      </c>
+      <c r="G14" s="4">
+        <v>219.0</v>
+      </c>
+      <c r="H14" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="5">
+        <v>4679.0</v>
+      </c>
+      <c r="E15" s="5">
+        <v>22.0</v>
+      </c>
+      <c r="F15" s="5">
+        <v>281.0</v>
+      </c>
+      <c r="G15" s="4">
+        <v>94.0</v>
+      </c>
+      <c r="H15" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="5">
+        <v>4957.0</v>
+      </c>
+      <c r="E16" s="5">
+        <v>93.0</v>
+      </c>
+      <c r="F16" s="5">
+        <v>276.0</v>
+      </c>
+      <c r="G16" s="4">
+        <v>397.0</v>
+      </c>
+      <c r="H16" s="6">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="5">
+        <v>2924.0</v>
+      </c>
+      <c r="E17" s="5">
+        <v>131.0</v>
+      </c>
+      <c r="F17" s="5">
+        <v>58.0</v>
+      </c>
+      <c r="G17" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="H17" s="6">
+        <v>7.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="5">
+        <v>7200.0</v>
+      </c>
+      <c r="E18" s="5">
+        <v>96.0</v>
+      </c>
+      <c r="F18" s="5">
+        <v>315.0</v>
+      </c>
+      <c r="G18" s="6">
+        <v>288.0</v>
+      </c>
+      <c r="H18" s="6">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="5">
+        <v>2177.0</v>
+      </c>
+      <c r="E19" s="5">
+        <v>23.0</v>
+      </c>
+      <c r="F19" s="5">
+        <v>262.0</v>
+      </c>
+      <c r="G19" s="6">
+        <v>131.0</v>
+      </c>
+      <c r="H19" s="6">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" s="5">
+        <v>4367.0</v>
+      </c>
+      <c r="E20" s="5">
+        <v>126.0</v>
+      </c>
+      <c r="F20" s="5">
+        <v>161.0</v>
+      </c>
+      <c r="G20" s="6">
+        <v>262.0</v>
+      </c>
+      <c r="H20" s="6">
+        <v>6.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2461,7 +3380,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2972,7 +3891,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -3372,7 +4291,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -3864,7 +4783,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -4314,7 +5233,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -4808,418 +5727,4 @@
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="18.38"/>
-    <col customWidth="1" min="2" max="2" width="18.0"/>
-    <col customWidth="1" min="3" max="3" width="14.88"/>
-    <col customWidth="1" min="4" max="4" width="18.25"/>
-    <col customWidth="1" min="5" max="5" width="80.5"/>
-    <col customWidth="1" min="6" max="6" width="15.13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E26" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F29" s="9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: TC08 dynamic header row detection using iterrows
</commit_message>
<xml_diff>
--- a/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
+++ b/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="122">
   <si>
     <t>date</t>
   </si>
@@ -375,6 +375,18 @@
   </si>
   <si>
     <t>Existen filas de informacion adicional agregadas por el usuario ejemplo "Comentarios de juan" las cuales no deben serconsideras, la informacion se encuentra completa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC_X — </t>
+  </si>
+  <si>
+    <t>Headers parcialmente en fila incorrecta</t>
+  </si>
+  <si>
+    <t>el archivo tiene algunos encabezados en una fila y otros en otra fila diferente. Comportamiento esperado: error crítico indicando estructura inválida.</t>
+  </si>
+  <si>
+    <t>Ejemplo el usuario tiene el dato date en A1 y el resto de datos en B2,C2,D2</t>
   </si>
 </sst>
 </file>
@@ -444,7 +456,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border/>
     <border>
       <left style="thin">
@@ -460,22 +472,11 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -525,9 +526,6 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="2" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1877,48 +1875,48 @@
         <v>75</v>
       </c>
       <c r="F6" s="16"/>
-      <c r="G6" s="17"/>
+      <c r="G6" s="16"/>
       <c r="H6" s="12"/>
       <c r="I6" s="12"/>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="18"/>
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
+      <c r="A7" s="17"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
       <c r="H7" s="12"/>
       <c r="I7" s="12"/>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="18"/>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="19"/>
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
       <c r="H8" s="12"/>
       <c r="I8" s="12"/>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="20"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
       <c r="H9" s="12"/>
       <c r="I9" s="12"/>
     </row>
@@ -1955,7 +1953,7 @@
       <c r="C11" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="D11" s="22"/>
+      <c r="D11" s="21"/>
       <c r="E11" s="13" t="s">
         <v>70</v>
       </c>
@@ -1967,227 +1965,241 @@
       <c r="I11" s="12"/>
     </row>
     <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="23" t="s">
+      <c r="A12" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="E12" s="23"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="24"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
     </row>
     <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="22" t="s">
         <v>95</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="E13" s="23"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
     </row>
     <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="C14" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="D14" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="E14" s="23"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
       <c r="H14" s="12"/>
       <c r="I14" s="12"/>
     </row>
     <row r="15" ht="22.5" customHeight="1">
-      <c r="A15" s="25"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
       <c r="H15" s="12"/>
       <c r="I15" s="12"/>
     </row>
     <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="25"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
+      <c r="A16" s="24"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
     </row>
     <row r="17" ht="22.5" customHeight="1">
-      <c r="A17" s="20" t="s">
+      <c r="A17" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="20" t="s">
+      <c r="D17" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
     </row>
     <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="27" t="s">
         <v>100</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="27" t="s">
         <v>101</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="E18" s="29"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="29"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
     </row>
     <row r="19" ht="22.5" customHeight="1">
-      <c r="A19" s="27" t="s">
+      <c r="A19" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="27" t="s">
         <v>103</v>
       </c>
-      <c r="C19" s="28" t="s">
+      <c r="C19" s="27" t="s">
         <v>104</v>
       </c>
-      <c r="D19" s="28" t="s">
+      <c r="D19" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="E19" s="29"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
     </row>
     <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="C20" s="28" t="s">
+      <c r="C20" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="D20" s="28" t="s">
+      <c r="D20" s="27" t="s">
         <v>108</v>
       </c>
-      <c r="E20" s="29"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
       <c r="H20" s="12"/>
       <c r="I20" s="12"/>
     </row>
     <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="27" t="s">
+      <c r="A21" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="C21" s="28" t="s">
+      <c r="C21" s="27" t="s">
         <v>110</v>
       </c>
-      <c r="D21" s="28" t="s">
+      <c r="D21" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="E21" s="29"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="30"/>
+      <c r="E21" s="28"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
       <c r="H21" s="12"/>
       <c r="I21" s="12"/>
     </row>
     <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="31" t="s">
+      <c r="A22" s="30" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="32" t="s">
+      <c r="B22" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="C22" s="32" t="s">
+      <c r="C22" s="31" t="s">
         <v>113</v>
       </c>
-      <c r="D22" s="28" t="s">
+      <c r="D22" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="E22" s="33"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="34"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="33"/>
     </row>
     <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="32" t="s">
+      <c r="A23" s="31" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="32" t="s">
+      <c r="B23" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="C23" s="32" t="s">
+      <c r="C23" s="31" t="s">
         <v>116</v>
       </c>
-      <c r="D23" s="28" t="s">
+      <c r="D23" s="27" t="s">
         <v>117</v>
       </c>
-      <c r="E23" s="33"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="34"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="33"/>
     </row>
     <row r="24" ht="22.5" customHeight="1">
-      <c r="A24" s="25"/>
-      <c r="B24" s="25"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="35"/>
-      <c r="G24" s="35"/>
+      <c r="A24" s="24"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="34"/>
     </row>
     <row r="26">
       <c r="C26" s="7"/>
     </row>
     <row r="27">
       <c r="B27" s="7"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>121</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -2581,133 +2593,69 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="6">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="1"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="1"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="1"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="5">
-        <v>5168.0</v>
-      </c>
-      <c r="E7" s="5">
-        <v>134.0</v>
-      </c>
-      <c r="F7" s="5">
-        <v>258.0</v>
-      </c>
-      <c r="G7" s="4">
-        <v>362.0</v>
-      </c>
-      <c r="H7" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="5">
-        <v>2314.0</v>
-      </c>
-      <c r="E8" s="5">
-        <v>26.0</v>
-      </c>
-      <c r="F8" s="5">
-        <v>162.0</v>
-      </c>
-      <c r="G8" s="4">
-        <v>46.0</v>
-      </c>
-      <c r="H8" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="5">
-        <v>3496.0</v>
-      </c>
-      <c r="E9" s="5">
-        <v>92.0</v>
-      </c>
-      <c r="F9" s="5">
-        <v>61.0</v>
-      </c>
-      <c r="G9" s="4">
-        <v>175.0</v>
-      </c>
-      <c r="H9" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="5">
-        <v>1790.0</v>
-      </c>
-      <c r="E10" s="5">
-        <v>87.0</v>
-      </c>
-      <c r="F10" s="5">
-        <v>370.0</v>
-      </c>
-      <c r="G10" s="4">
-        <v>54.0</v>
-      </c>
-      <c r="H10" s="6">
-        <v>4.0</v>
       </c>
     </row>
     <row r="11">
@@ -2718,22 +2666,22 @@
         <v>8</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D11" s="5">
-        <v>9764.0</v>
+        <v>5168.0</v>
       </c>
       <c r="E11" s="5">
-        <v>53.0</v>
+        <v>134.0</v>
       </c>
       <c r="F11" s="5">
-        <v>118.0</v>
+        <v>258.0</v>
       </c>
       <c r="G11" s="4">
-        <v>293.0</v>
+        <v>362.0</v>
       </c>
       <c r="H11" s="6">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="12">
@@ -2744,19 +2692,19 @@
         <v>8</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D12" s="5">
-        <v>2912.0</v>
+        <v>2314.0</v>
       </c>
       <c r="E12" s="5">
         <v>26.0</v>
       </c>
       <c r="F12" s="5">
-        <v>187.0</v>
+        <v>162.0</v>
       </c>
       <c r="G12" s="4">
-        <v>204.0</v>
+        <v>46.0</v>
       </c>
       <c r="H12" s="6">
         <v>1.0</v>
@@ -2770,19 +2718,19 @@
         <v>8</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D13" s="5">
-        <v>4736.0</v>
+        <v>3496.0</v>
       </c>
       <c r="E13" s="5">
-        <v>123.0</v>
+        <v>92.0</v>
       </c>
       <c r="F13" s="5">
-        <v>198.0</v>
+        <v>61.0</v>
       </c>
       <c r="G13" s="4">
-        <v>237.0</v>
+        <v>175.0</v>
       </c>
       <c r="H13" s="6">
         <v>1.0</v>
@@ -2793,22 +2741,22 @@
         <v>45658.0</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D14" s="5">
-        <v>7311.0</v>
+        <v>1790.0</v>
       </c>
       <c r="E14" s="5">
-        <v>149.0</v>
+        <v>87.0</v>
       </c>
       <c r="F14" s="5">
-        <v>230.0</v>
+        <v>370.0</v>
       </c>
       <c r="G14" s="4">
-        <v>219.0</v>
+        <v>54.0</v>
       </c>
       <c r="H14" s="6">
         <v>4.0</v>
@@ -2819,25 +2767,25 @@
         <v>45658.0</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D15" s="5">
-        <v>4679.0</v>
+        <v>9764.0</v>
       </c>
       <c r="E15" s="5">
-        <v>22.0</v>
+        <v>53.0</v>
       </c>
       <c r="F15" s="5">
-        <v>281.0</v>
+        <v>118.0</v>
       </c>
       <c r="G15" s="4">
-        <v>94.0</v>
+        <v>293.0</v>
       </c>
       <c r="H15" s="6">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="16">
@@ -2845,25 +2793,25 @@
         <v>45658.0</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D16" s="5">
-        <v>4957.0</v>
+        <v>2912.0</v>
       </c>
       <c r="E16" s="5">
-        <v>93.0</v>
+        <v>26.0</v>
       </c>
       <c r="F16" s="5">
-        <v>276.0</v>
+        <v>187.0</v>
       </c>
       <c r="G16" s="4">
-        <v>397.0</v>
+        <v>204.0</v>
       </c>
       <c r="H16" s="6">
-        <v>5.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="17">
@@ -2871,102 +2819,206 @@
         <v>45658.0</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D17" s="5">
-        <v>2924.0</v>
+        <v>4736.0</v>
       </c>
       <c r="E17" s="5">
-        <v>131.0</v>
+        <v>123.0</v>
       </c>
       <c r="F17" s="5">
-        <v>58.0</v>
+        <v>198.0</v>
       </c>
       <c r="G17" s="4">
-        <v>175.0</v>
+        <v>237.0</v>
       </c>
       <c r="H17" s="6">
-        <v>7.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4">
         <v>45658.0</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>13</v>
+      <c r="B18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D18" s="5">
-        <v>7200.0</v>
+        <v>7311.0</v>
       </c>
       <c r="E18" s="5">
-        <v>96.0</v>
+        <v>149.0</v>
       </c>
       <c r="F18" s="5">
-        <v>315.0</v>
-      </c>
-      <c r="G18" s="6">
-        <v>288.0</v>
+        <v>230.0</v>
+      </c>
+      <c r="G18" s="4">
+        <v>219.0</v>
       </c>
       <c r="H18" s="6">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4">
         <v>45658.0</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>14</v>
+      <c r="B19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="D19" s="5">
-        <v>2177.0</v>
+        <v>4679.0</v>
       </c>
       <c r="E19" s="5">
-        <v>23.0</v>
+        <v>22.0</v>
       </c>
       <c r="F19" s="5">
-        <v>262.0</v>
-      </c>
-      <c r="G19" s="6">
-        <v>131.0</v>
+        <v>281.0</v>
+      </c>
+      <c r="G19" s="4">
+        <v>94.0</v>
       </c>
       <c r="H19" s="6">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4">
         <v>45658.0</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C20" s="3" t="s">
+      <c r="B20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="5">
+        <v>4957.0</v>
+      </c>
+      <c r="E20" s="5">
+        <v>93.0</v>
+      </c>
+      <c r="F20" s="5">
+        <v>276.0</v>
+      </c>
+      <c r="G20" s="4">
+        <v>397.0</v>
+      </c>
+      <c r="H20" s="6">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="5">
+        <v>2924.0</v>
+      </c>
+      <c r="E21" s="5">
+        <v>131.0</v>
+      </c>
+      <c r="F21" s="5">
+        <v>58.0</v>
+      </c>
+      <c r="G21" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="H21" s="6">
+        <v>7.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="5">
+        <v>7200.0</v>
+      </c>
+      <c r="E22" s="5">
+        <v>96.0</v>
+      </c>
+      <c r="F22" s="5">
+        <v>315.0</v>
+      </c>
+      <c r="G22" s="6">
+        <v>288.0</v>
+      </c>
+      <c r="H22" s="6">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="5">
+        <v>2177.0</v>
+      </c>
+      <c r="E23" s="5">
+        <v>23.0</v>
+      </c>
+      <c r="F23" s="5">
+        <v>262.0</v>
+      </c>
+      <c r="G23" s="6">
+        <v>131.0</v>
+      </c>
+      <c r="H23" s="6">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D24" s="5">
         <v>4367.0</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E24" s="5">
         <v>126.0</v>
       </c>
-      <c r="F20" s="5">
+      <c r="F24" s="5">
         <v>161.0</v>
       </c>
-      <c r="G20" s="6">
+      <c r="G24" s="6">
         <v>262.0</v>
       </c>
-      <c r="H20" s="6">
+      <c r="H24" s="6">
         <v>6.0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add Unnamed columns cleanup after second Excel read
</commit_message>
<xml_diff>
--- a/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
+++ b/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
@@ -4,16 +4,18 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="TC01" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="EX1" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="TC02" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="TC03" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="TC04" sheetId="5" r:id="rId9"/>
-    <sheet state="visible" name="TC05" sheetId="6" r:id="rId10"/>
-    <sheet state="visible" name="TC06" sheetId="7" r:id="rId11"/>
-    <sheet state="visible" name="TC07" sheetId="8" r:id="rId12"/>
-    <sheet state="visible" name="TC08" sheetId="9" r:id="rId13"/>
-    <sheet state="visible" name="Hoja 12" sheetId="10" r:id="rId14"/>
-    <sheet state="visible" name="TC Codigo" sheetId="11" r:id="rId15"/>
+    <sheet state="visible" name="Jun" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="EX1" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="TC02" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="TC03" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="TC04" sheetId="6" r:id="rId10"/>
+    <sheet state="visible" name="TC05" sheetId="7" r:id="rId11"/>
+    <sheet state="visible" name="TC06" sheetId="8" r:id="rId12"/>
+    <sheet state="visible" name="TC07" sheetId="9" r:id="rId13"/>
+    <sheet state="visible" name="TC08" sheetId="10" r:id="rId14"/>
+    <sheet state="visible" name="Hoja 12" sheetId="11" r:id="rId15"/>
+    <sheet state="visible" name="TC Codigo" sheetId="12" r:id="rId16"/>
+    <sheet state="visible" name="EX2" sheetId="13" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -21,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="122">
   <si>
     <t>date</t>
   </si>
@@ -311,7 +313,7 @@
     <t>Lo encabezados comienzan la columna 1 pero desface en horizontal</t>
   </si>
   <si>
-    <t xml:space="preserve">La columna de informacion requerida se encuentra completa pero enpieza en D1 es decir se A1 a C1 no vontine ningun tipo de dato y es basura </t>
+    <t xml:space="preserve">La columna de informacion requerida se encuentra completa pero enpieza en D1 es decir se A1 a C1 no contine ningun tipo de dato y es basura </t>
   </si>
   <si>
     <t>Desface de Columnas y Filas</t>
@@ -418,7 +420,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -447,12 +449,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF1C232"/>
         <bgColor rgb="FFF1C232"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCC0000"/>
-        <bgColor rgb="FFCC0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -543,10 +539,10 @@
     <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -661,6 +657,14 @@
 </file>
 
 <file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -1325,6 +1329,502 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
+    <col customWidth="1" min="3" max="3" width="21.63"/>
+    <col customWidth="1" min="14" max="15" width="24.38"/>
+  </cols>
+  <sheetData>
+    <row r="6">
+      <c r="A6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J6" s="3"/>
+      <c r="K6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>362.0</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5">
+        <v>5168.0</v>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5">
+        <v>134.0</v>
+      </c>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5">
+        <v>258.0</v>
+      </c>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <v>46.0</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5">
+        <v>2314.0</v>
+      </c>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5">
+        <v>162.0</v>
+      </c>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5">
+        <v>3496.0</v>
+      </c>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5">
+        <v>92.0</v>
+      </c>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5">
+        <v>61.0</v>
+      </c>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4">
+        <v>54.0</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5">
+        <v>1790.0</v>
+      </c>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5">
+        <v>87.0</v>
+      </c>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5">
+        <v>370.0</v>
+      </c>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4">
+        <v>293.0</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5">
+        <v>9764.0</v>
+      </c>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5">
+        <v>53.0</v>
+      </c>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5">
+        <v>118.0</v>
+      </c>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4">
+        <v>204.0</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5">
+        <v>2912.0</v>
+      </c>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5">
+        <v>187.0</v>
+      </c>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4">
+        <v>237.0</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5">
+        <v>4736.0</v>
+      </c>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5">
+        <v>123.0</v>
+      </c>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5">
+        <v>198.0</v>
+      </c>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <v>219.0</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5">
+        <v>7311.0</v>
+      </c>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5">
+        <v>149.0</v>
+      </c>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5">
+        <v>230.0</v>
+      </c>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4">
+        <v>94.0</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5">
+        <v>4679.0</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5">
+        <v>22.0</v>
+      </c>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5">
+        <v>281.0</v>
+      </c>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4">
+        <v>397.0</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5">
+        <v>4957.0</v>
+      </c>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5">
+        <v>93.0</v>
+      </c>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5">
+        <v>276.0</v>
+      </c>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L16" s="6"/>
+      <c r="M16" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5">
+        <v>2924.0</v>
+      </c>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5">
+        <v>131.0</v>
+      </c>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5">
+        <v>58.0</v>
+      </c>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="N17" s="2"/>
+      <c r="O17" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6">
+        <v>288.0</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5">
+        <v>7200.0</v>
+      </c>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5">
+        <v>96.0</v>
+      </c>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5">
+        <v>315.0</v>
+      </c>
+      <c r="J18" s="6"/>
+      <c r="K18" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L18" s="6"/>
+      <c r="M18" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="N18" s="3"/>
+      <c r="O18" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6">
+        <v>131.0</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5">
+        <v>2177.0</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5">
+        <v>23.0</v>
+      </c>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5">
+        <v>262.0</v>
+      </c>
+      <c r="J19" s="6"/>
+      <c r="K19" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L19" s="6"/>
+      <c r="M19" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="N19" s="3"/>
+      <c r="O19" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6">
+        <v>262.0</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5">
+        <v>4367.0</v>
+      </c>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5">
+        <v>126.0</v>
+      </c>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5">
+        <v>161.0</v>
+      </c>
+      <c r="J20" s="6"/>
+      <c r="K20" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="L20" s="6"/>
+      <c r="M20" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="N20" s="3"/>
+      <c r="O20" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
     <col customWidth="1" min="1" max="1" width="18.38"/>
     <col customWidth="1" min="2" max="2" width="18.0"/>
     <col customWidth="1" min="3" max="3" width="14.88"/>
@@ -1732,7 +2232,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -1965,21 +2465,23 @@
       <c r="I11" s="12"/>
     </row>
     <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="E12" s="22"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
+      <c r="E12" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
     </row>
@@ -2206,6 +2708,723 @@
   <tableParts count="1">
     <tablePart r:id="rId3"/>
   </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="F1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="O1" s="3"/>
+      <c r="P1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="F2" s="4">
+        <v>362.0</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5">
+        <v>5168.0</v>
+      </c>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5">
+        <v>134.0</v>
+      </c>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5">
+        <v>258.0</v>
+      </c>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="F3" s="4">
+        <v>46.0</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5">
+        <v>2314.0</v>
+      </c>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5">
+        <v>162.0</v>
+      </c>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="F4" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5">
+        <v>3496.0</v>
+      </c>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5">
+        <v>92.0</v>
+      </c>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5">
+        <v>61.0</v>
+      </c>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="F5" s="4">
+        <v>54.0</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5">
+        <v>1790.0</v>
+      </c>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5">
+        <v>87.0</v>
+      </c>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5">
+        <v>370.0</v>
+      </c>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="F6" s="4">
+        <v>293.0</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5">
+        <v>9764.0</v>
+      </c>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5">
+        <v>53.0</v>
+      </c>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5">
+        <v>118.0</v>
+      </c>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="F7" s="4">
+        <v>204.0</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5">
+        <v>2912.0</v>
+      </c>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5">
+        <v>187.0</v>
+      </c>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="F8" s="4">
+        <v>237.0</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5">
+        <v>4736.0</v>
+      </c>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5">
+        <v>123.0</v>
+      </c>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5">
+        <v>198.0</v>
+      </c>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="S8" s="2"/>
+      <c r="T8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="F9" s="4">
+        <v>219.0</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5">
+        <v>7311.0</v>
+      </c>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5">
+        <v>149.0</v>
+      </c>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5">
+        <v>230.0</v>
+      </c>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="S9" s="2"/>
+      <c r="T9" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="F10" s="4">
+        <v>94.0</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5">
+        <v>4679.0</v>
+      </c>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5">
+        <v>22.0</v>
+      </c>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5">
+        <v>281.0</v>
+      </c>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="S10" s="2"/>
+      <c r="T10" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="F11" s="4">
+        <v>397.0</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5">
+        <v>4957.0</v>
+      </c>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5">
+        <v>93.0</v>
+      </c>
+      <c r="M11" s="5"/>
+      <c r="N11" s="5">
+        <v>276.0</v>
+      </c>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="S11" s="2"/>
+      <c r="T11" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="F12" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5">
+        <v>2924.0</v>
+      </c>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5">
+        <v>131.0</v>
+      </c>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5">
+        <v>58.0</v>
+      </c>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="S12" s="2"/>
+      <c r="T12" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="F13" s="6">
+        <v>288.0</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5">
+        <v>7200.0</v>
+      </c>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5">
+        <v>96.0</v>
+      </c>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5">
+        <v>315.0</v>
+      </c>
+      <c r="O13" s="6"/>
+      <c r="P13" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="S13" s="3"/>
+      <c r="T13" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="F14" s="6">
+        <v>131.0</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5">
+        <v>2177.0</v>
+      </c>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5">
+        <v>23.0</v>
+      </c>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5">
+        <v>262.0</v>
+      </c>
+      <c r="O14" s="6"/>
+      <c r="P14" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="S14" s="3"/>
+      <c r="T14" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="E15" s="3"/>
+      <c r="F15" s="6">
+        <v>262.0</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5">
+        <v>4367.0</v>
+      </c>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5">
+        <v>126.0</v>
+      </c>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5">
+        <v>161.0</v>
+      </c>
+      <c r="O15" s="6"/>
+      <c r="P15" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="S15" s="3"/>
+      <c r="T15" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" s="4"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="6"/>
+      <c r="Q16" s="6"/>
+      <c r="R16" s="2"/>
+      <c r="S16" s="2"/>
+    </row>
+    <row r="17">
+      <c r="E17" s="4"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="6"/>
+      <c r="Q17" s="6"/>
+      <c r="R17" s="2"/>
+      <c r="S17" s="2"/>
+    </row>
+    <row r="18">
+      <c r="E18" s="4"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="6"/>
+      <c r="Q18" s="6"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
+    </row>
+    <row r="19">
+      <c r="E19" s="4"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="6"/>
+      <c r="Q19" s="6"/>
+      <c r="R19" s="2"/>
+      <c r="S19" s="2"/>
+    </row>
+    <row r="20">
+      <c r="E20" s="4"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="6"/>
+      <c r="Q20" s="6"/>
+      <c r="R20" s="2"/>
+      <c r="S20" s="2"/>
+    </row>
+    <row r="21">
+      <c r="E21" s="4"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="6"/>
+      <c r="Q21" s="6"/>
+      <c r="R21" s="2"/>
+      <c r="S21" s="2"/>
+    </row>
+    <row r="22">
+      <c r="E22" s="4"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="6"/>
+      <c r="Q22" s="6"/>
+      <c r="R22" s="2"/>
+      <c r="S22" s="2"/>
+    </row>
+    <row r="23">
+      <c r="E23" s="4"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
+      <c r="P23" s="6"/>
+      <c r="Q23" s="6"/>
+      <c r="R23" s="2"/>
+      <c r="S23" s="2"/>
+    </row>
+    <row r="24">
+      <c r="E24" s="4"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="6"/>
+      <c r="Q24" s="6"/>
+      <c r="R24" s="2"/>
+      <c r="S24" s="2"/>
+    </row>
+    <row r="25">
+      <c r="E25" s="4"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="6"/>
+      <c r="Q25" s="6"/>
+      <c r="R25" s="2"/>
+      <c r="S25" s="2"/>
+    </row>
+    <row r="26">
+      <c r="E26" s="4"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+      <c r="L26" s="5"/>
+      <c r="M26" s="5"/>
+      <c r="N26" s="4"/>
+      <c r="O26" s="4"/>
+      <c r="P26" s="6"/>
+      <c r="Q26" s="6"/>
+      <c r="R26" s="2"/>
+      <c r="S26" s="2"/>
+    </row>
+    <row r="27">
+      <c r="E27" s="6"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+      <c r="L27" s="5"/>
+      <c r="M27" s="5"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="4"/>
+      <c r="P27" s="6"/>
+      <c r="Q27" s="6"/>
+      <c r="R27" s="3"/>
+      <c r="S27" s="3"/>
+    </row>
+    <row r="28">
+      <c r="E28" s="6"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+      <c r="L28" s="5"/>
+      <c r="M28" s="5"/>
+      <c r="N28" s="6"/>
+      <c r="O28" s="4"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="6"/>
+      <c r="R28" s="3"/>
+      <c r="S28" s="3"/>
+    </row>
+    <row r="29">
+      <c r="E29" s="6"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="6"/>
+      <c r="O29" s="4"/>
+      <c r="P29" s="6"/>
+      <c r="Q29" s="6"/>
+      <c r="R29" s="3"/>
+      <c r="S29" s="3"/>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2217,366 +3436,392 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="D2" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="5">
+      <c r="G2" s="5">
         <v>5168.0</v>
       </c>
-      <c r="E1" s="5">
+      <c r="H2" s="5">
         <v>134.0</v>
       </c>
-      <c r="F1" s="5">
+      <c r="I2" s="5">
         <v>258.0</v>
       </c>
-      <c r="G1" s="4">
+      <c r="J2" s="4">
         <v>362.0</v>
       </c>
-      <c r="H1" s="6">
+      <c r="K2" s="6">
         <v>4.0</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2" t="s">
+    <row r="3">
+      <c r="D3" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="5">
+      <c r="G3" s="5">
         <v>2314.0</v>
       </c>
-      <c r="E2" s="5">
+      <c r="H3" s="5">
         <v>26.0</v>
       </c>
-      <c r="F2" s="5">
+      <c r="I3" s="5">
         <v>162.0</v>
       </c>
-      <c r="G2" s="4">
+      <c r="J3" s="4">
         <v>46.0</v>
       </c>
-      <c r="H2" s="6">
+      <c r="K3" s="6">
         <v>1.0</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2" t="s">
+    <row r="4">
+      <c r="D4" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="5">
+      <c r="G4" s="5">
         <v>3496.0</v>
       </c>
-      <c r="E3" s="5">
+      <c r="H4" s="5">
         <v>92.0</v>
       </c>
-      <c r="F3" s="5">
+      <c r="I4" s="5">
         <v>61.0</v>
       </c>
-      <c r="G3" s="4">
+      <c r="J4" s="4">
         <v>175.0</v>
       </c>
-      <c r="H3" s="6">
+      <c r="K4" s="6">
         <v>1.0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
+    <row r="5">
+      <c r="D5" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="5">
+      <c r="G5" s="5">
         <v>1790.0</v>
       </c>
-      <c r="E4" s="5">
+      <c r="H5" s="5">
         <v>87.0</v>
       </c>
-      <c r="F4" s="5">
+      <c r="I5" s="5">
         <v>370.0</v>
       </c>
-      <c r="G4" s="4">
+      <c r="J5" s="4">
         <v>54.0</v>
       </c>
-      <c r="H4" s="6">
+      <c r="K5" s="6">
         <v>4.0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="2" t="s">
+    <row r="6">
+      <c r="D6" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="5">
+      <c r="G6" s="5">
         <v>9764.0</v>
       </c>
-      <c r="E5" s="5">
+      <c r="H6" s="5">
         <v>53.0</v>
       </c>
-      <c r="F5" s="5">
+      <c r="I6" s="5">
         <v>118.0</v>
       </c>
-      <c r="G5" s="4">
+      <c r="J6" s="4">
         <v>293.0</v>
       </c>
-      <c r="H5" s="6">
+      <c r="K6" s="6">
         <v>3.0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="2" t="s">
+    <row r="7">
+      <c r="D7" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="5">
+      <c r="G7" s="5">
         <v>2912.0</v>
       </c>
-      <c r="E6" s="5">
+      <c r="H7" s="5">
         <v>26.0</v>
       </c>
-      <c r="F6" s="5">
+      <c r="I7" s="5">
         <v>187.0</v>
       </c>
-      <c r="G6" s="4">
+      <c r="J7" s="4">
         <v>204.0</v>
       </c>
-      <c r="H6" s="6">
+      <c r="K7" s="6">
         <v>1.0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="2" t="s">
+    <row r="8">
+      <c r="D8" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="5">
+      <c r="G8" s="5">
         <v>4736.0</v>
       </c>
-      <c r="E7" s="5">
+      <c r="H8" s="5">
         <v>123.0</v>
       </c>
-      <c r="F7" s="5">
+      <c r="I8" s="5">
         <v>198.0</v>
       </c>
-      <c r="G7" s="4">
+      <c r="J8" s="4">
         <v>237.0</v>
       </c>
-      <c r="H7" s="6">
+      <c r="K8" s="6">
         <v>1.0</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="2" t="s">
+    <row r="9">
+      <c r="D9" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="5">
+      <c r="G9" s="5">
         <v>7311.0</v>
       </c>
-      <c r="E8" s="5">
+      <c r="H9" s="5">
         <v>149.0</v>
       </c>
-      <c r="F8" s="5">
+      <c r="I9" s="5">
         <v>230.0</v>
       </c>
-      <c r="G8" s="4">
+      <c r="J9" s="4">
         <v>219.0</v>
       </c>
-      <c r="H8" s="6">
+      <c r="K9" s="6">
         <v>4.0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="2" t="s">
+    <row r="10">
+      <c r="D10" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="5">
+      <c r="G10" s="5">
         <v>4679.0</v>
       </c>
-      <c r="E9" s="5">
+      <c r="H10" s="5">
         <v>22.0</v>
       </c>
-      <c r="F9" s="5">
+      <c r="I10" s="5">
         <v>281.0</v>
       </c>
-      <c r="G9" s="4">
+      <c r="J10" s="4">
         <v>94.0</v>
       </c>
-      <c r="H9" s="6">
+      <c r="K10" s="6">
         <v>1.0</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="2" t="s">
+    <row r="11">
+      <c r="D11" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="5">
+      <c r="G11" s="5">
         <v>4957.0</v>
       </c>
-      <c r="E10" s="5">
+      <c r="H11" s="5">
         <v>93.0</v>
       </c>
-      <c r="F10" s="5">
+      <c r="I11" s="5">
         <v>276.0</v>
       </c>
-      <c r="G10" s="4">
+      <c r="J11" s="4">
         <v>397.0</v>
       </c>
-      <c r="H10" s="6">
+      <c r="K11" s="6">
         <v>5.0</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="2" t="s">
+    <row r="12">
+      <c r="D12" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="5">
+      <c r="G12" s="5">
         <v>2924.0</v>
       </c>
-      <c r="E11" s="5">
+      <c r="H12" s="5">
         <v>131.0</v>
       </c>
-      <c r="F11" s="5">
+      <c r="I12" s="5">
         <v>58.0</v>
       </c>
-      <c r="G11" s="4">
+      <c r="J12" s="4">
         <v>175.0</v>
       </c>
-      <c r="H11" s="6">
+      <c r="K12" s="6">
         <v>7.0</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="3" t="s">
+    <row r="13">
+      <c r="D13" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="5">
+      <c r="G13" s="5">
         <v>7200.0</v>
       </c>
-      <c r="E12" s="5">
+      <c r="H13" s="5">
         <v>96.0</v>
       </c>
-      <c r="F12" s="5">
+      <c r="I13" s="5">
         <v>315.0</v>
       </c>
-      <c r="G12" s="6">
+      <c r="J13" s="6">
         <v>288.0</v>
       </c>
-      <c r="H12" s="6">
+      <c r="K13" s="6">
         <v>2.0</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="3" t="s">
+    <row r="14">
+      <c r="D14" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="5">
+      <c r="G14" s="5">
         <v>2177.0</v>
       </c>
-      <c r="E13" s="5">
+      <c r="H14" s="5">
         <v>23.0</v>
       </c>
-      <c r="F13" s="5">
+      <c r="I14" s="5">
         <v>262.0</v>
       </c>
-      <c r="G13" s="6">
+      <c r="J14" s="6">
         <v>131.0</v>
       </c>
-      <c r="H13" s="6">
+      <c r="K14" s="6">
         <v>0.0</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="3" t="s">
+    <row r="15">
+      <c r="D15" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="5">
+      <c r="G15" s="5">
         <v>4367.0</v>
       </c>
-      <c r="E14" s="5">
+      <c r="H15" s="5">
         <v>126.0</v>
       </c>
-      <c r="F14" s="5">
+      <c r="I15" s="5">
         <v>161.0</v>
       </c>
-      <c r="G14" s="6">
+      <c r="J15" s="6">
         <v>262.0</v>
       </c>
-      <c r="H14" s="6">
+      <c r="K15" s="6">
         <v>6.0</v>
       </c>
     </row>
@@ -2586,6 +3831,638 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="6"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="4"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="6"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="6"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="6"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="6"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="6"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="6"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+    </row>
+    <row r="16">
+      <c r="D16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="M16" s="3"/>
+      <c r="N16" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q16" s="2"/>
+      <c r="R16" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="D17" s="4">
+        <v>362.0</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5">
+        <v>5168.0</v>
+      </c>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5">
+        <v>134.0</v>
+      </c>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5">
+        <v>258.0</v>
+      </c>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O17" s="6"/>
+      <c r="P17" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="D18" s="4">
+        <v>46.0</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5">
+        <v>2314.0</v>
+      </c>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5">
+        <v>162.0</v>
+      </c>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O18" s="6"/>
+      <c r="P18" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="D19" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5">
+        <v>3496.0</v>
+      </c>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5">
+        <v>92.0</v>
+      </c>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5">
+        <v>61.0</v>
+      </c>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O19" s="6"/>
+      <c r="P19" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" s="4">
+        <v>54.0</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5">
+        <v>1790.0</v>
+      </c>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5">
+        <v>87.0</v>
+      </c>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5">
+        <v>370.0</v>
+      </c>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O20" s="6"/>
+      <c r="P20" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="D21" s="4">
+        <v>293.0</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5">
+        <v>9764.0</v>
+      </c>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5">
+        <v>53.0</v>
+      </c>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5">
+        <v>118.0</v>
+      </c>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O21" s="6"/>
+      <c r="P21" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="Q21" s="2"/>
+      <c r="R21" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="D22" s="4">
+        <v>204.0</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5">
+        <v>2912.0</v>
+      </c>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="K22" s="5"/>
+      <c r="L22" s="5">
+        <v>187.0</v>
+      </c>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O22" s="6"/>
+      <c r="P22" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="Q22" s="2"/>
+      <c r="R22" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="D23" s="4">
+        <v>237.0</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5">
+        <v>4736.0</v>
+      </c>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5">
+        <v>123.0</v>
+      </c>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5">
+        <v>198.0</v>
+      </c>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="Q23" s="2"/>
+      <c r="R23" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="D24" s="4">
+        <v>219.0</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5">
+        <v>7311.0</v>
+      </c>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5">
+        <v>149.0</v>
+      </c>
+      <c r="K24" s="5"/>
+      <c r="L24" s="5">
+        <v>230.0</v>
+      </c>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O24" s="6"/>
+      <c r="P24" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="Q24" s="2"/>
+      <c r="R24" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="D25" s="4">
+        <v>94.0</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5">
+        <v>4679.0</v>
+      </c>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5">
+        <v>22.0</v>
+      </c>
+      <c r="K25" s="5"/>
+      <c r="L25" s="5">
+        <v>281.0</v>
+      </c>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O25" s="6"/>
+      <c r="P25" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="Q25" s="2"/>
+      <c r="R25" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" s="4">
+        <v>397.0</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5">
+        <v>4957.0</v>
+      </c>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5">
+        <v>93.0</v>
+      </c>
+      <c r="K26" s="5"/>
+      <c r="L26" s="5">
+        <v>276.0</v>
+      </c>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O26" s="6"/>
+      <c r="P26" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="Q26" s="2"/>
+      <c r="R26" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="D27" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5">
+        <v>2924.0</v>
+      </c>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5">
+        <v>131.0</v>
+      </c>
+      <c r="K27" s="5"/>
+      <c r="L27" s="5">
+        <v>58.0</v>
+      </c>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O27" s="6"/>
+      <c r="P27" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="Q27" s="2"/>
+      <c r="R27" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" s="6">
+        <v>288.0</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5">
+        <v>7200.0</v>
+      </c>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5">
+        <v>96.0</v>
+      </c>
+      <c r="K28" s="5"/>
+      <c r="L28" s="5">
+        <v>315.0</v>
+      </c>
+      <c r="M28" s="6"/>
+      <c r="N28" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O28" s="6"/>
+      <c r="P28" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="Q28" s="3"/>
+      <c r="R28" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="D29" s="6">
+        <v>131.0</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5">
+        <v>2177.0</v>
+      </c>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5">
+        <v>23.0</v>
+      </c>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5">
+        <v>262.0</v>
+      </c>
+      <c r="M29" s="6"/>
+      <c r="N29" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O29" s="6"/>
+      <c r="P29" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="Q29" s="3"/>
+      <c r="R29" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="D30" s="6">
+        <v>262.0</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G30" s="5"/>
+      <c r="H30" s="5">
+        <v>4367.0</v>
+      </c>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5">
+        <v>126.0</v>
+      </c>
+      <c r="K30" s="5"/>
+      <c r="L30" s="5">
+        <v>161.0</v>
+      </c>
+      <c r="M30" s="6"/>
+      <c r="N30" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="O30" s="6"/>
+      <c r="P30" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="Q30" s="3"/>
+      <c r="R30" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -3027,7 +4904,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -3432,7 +5309,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -3943,7 +5820,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -4343,7 +6220,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -4835,7 +6712,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -5283,500 +7160,4 @@
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <cols>
-    <col customWidth="1" min="3" max="3" width="21.63"/>
-    <col customWidth="1" min="14" max="15" width="24.38"/>
-  </cols>
-  <sheetData>
-    <row r="6">
-      <c r="A6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="J6" s="3"/>
-      <c r="K6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4">
-        <v>362.0</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5">
-        <v>5168.0</v>
-      </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5">
-        <v>134.0</v>
-      </c>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5">
-        <v>258.0</v>
-      </c>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4">
-        <v>46.0</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5">
-        <v>2314.0</v>
-      </c>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5">
-        <v>26.0</v>
-      </c>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5">
-        <v>162.0</v>
-      </c>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4">
-        <v>175.0</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5">
-        <v>3496.0</v>
-      </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5">
-        <v>92.0</v>
-      </c>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5">
-        <v>61.0</v>
-      </c>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4">
-        <v>54.0</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5">
-        <v>1790.0</v>
-      </c>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5">
-        <v>87.0</v>
-      </c>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5">
-        <v>370.0</v>
-      </c>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4">
-        <v>293.0</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5">
-        <v>9764.0</v>
-      </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5">
-        <v>53.0</v>
-      </c>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5">
-        <v>118.0</v>
-      </c>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4">
-        <v>204.0</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5">
-        <v>2912.0</v>
-      </c>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5">
-        <v>26.0</v>
-      </c>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5">
-        <v>187.0</v>
-      </c>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4">
-        <v>237.0</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5">
-        <v>4736.0</v>
-      </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5">
-        <v>123.0</v>
-      </c>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5">
-        <v>198.0</v>
-      </c>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4">
-        <v>219.0</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5">
-        <v>7311.0</v>
-      </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5">
-        <v>149.0</v>
-      </c>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5">
-        <v>230.0</v>
-      </c>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4">
-        <v>94.0</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5">
-        <v>4679.0</v>
-      </c>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5">
-        <v>22.0</v>
-      </c>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5">
-        <v>281.0</v>
-      </c>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4">
-        <v>397.0</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5">
-        <v>4957.0</v>
-      </c>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5">
-        <v>93.0</v>
-      </c>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5">
-        <v>276.0</v>
-      </c>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L16" s="6"/>
-      <c r="M16" s="6">
-        <v>5.0</v>
-      </c>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4">
-        <v>175.0</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5">
-        <v>2924.0</v>
-      </c>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5">
-        <v>131.0</v>
-      </c>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5">
-        <v>58.0</v>
-      </c>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L17" s="6"/>
-      <c r="M17" s="6">
-        <v>7.0</v>
-      </c>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6">
-        <v>288.0</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5">
-        <v>7200.0</v>
-      </c>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5">
-        <v>96.0</v>
-      </c>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5">
-        <v>315.0</v>
-      </c>
-      <c r="J18" s="6"/>
-      <c r="K18" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6">
-        <v>2.0</v>
-      </c>
-      <c r="N18" s="3"/>
-      <c r="O18" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6">
-        <v>131.0</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5">
-        <v>2177.0</v>
-      </c>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5">
-        <v>23.0</v>
-      </c>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5">
-        <v>262.0</v>
-      </c>
-      <c r="J19" s="6"/>
-      <c r="K19" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L19" s="6"/>
-      <c r="M19" s="6">
-        <v>0.0</v>
-      </c>
-      <c r="N19" s="3"/>
-      <c r="O19" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6">
-        <v>262.0</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5">
-        <v>4367.0</v>
-      </c>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5">
-        <v>126.0</v>
-      </c>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5">
-        <v>161.0</v>
-      </c>
-      <c r="J20" s="6"/>
-      <c r="K20" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="L20" s="6"/>
-      <c r="M20" s="6">
-        <v>6.0</v>
-      </c>
-      <c r="N20" s="3"/>
-      <c r="O20" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated TC12 to address vertical offset gap; added new successful test cases TC12B and TC12C
</commit_message>
<xml_diff>
--- a/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
+++ b/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
@@ -10,11 +10,14 @@
     <sheet state="visible" name="TC10" sheetId="5" r:id="rId9"/>
     <sheet state="visible" name="TC11" sheetId="6" r:id="rId10"/>
     <sheet state="visible" name="TC12" sheetId="7" r:id="rId11"/>
-    <sheet state="visible" name="TC13" sheetId="8" r:id="rId12"/>
-    <sheet state="visible" name="TC14" sheetId="9" r:id="rId13"/>
-    <sheet state="visible" name="TC15" sheetId="10" r:id="rId14"/>
-    <sheet state="visible" name="Hoja 12" sheetId="11" r:id="rId15"/>
-    <sheet state="visible" name="TC Codigo" sheetId="12" r:id="rId16"/>
+    <sheet state="visible" name="TC12B" sheetId="8" r:id="rId12"/>
+    <sheet state="visible" name="TC12C" sheetId="9" r:id="rId13"/>
+    <sheet state="visible" name="TC13" sheetId="10" r:id="rId14"/>
+    <sheet state="visible" name="TC14" sheetId="11" r:id="rId15"/>
+    <sheet state="visible" name="TC15" sheetId="12" r:id="rId16"/>
+    <sheet state="visible" name="TC16" sheetId="13" r:id="rId17"/>
+    <sheet state="visible" name="Hoja 12" sheetId="14" r:id="rId18"/>
+    <sheet state="visible" name="TC Codigo" sheetId="15" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -22,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="187">
   <si>
     <t>date</t>
   </si>
@@ -330,7 +333,7 @@
     <t xml:space="preserve">El programa debe indicar que los header se encuentran completos </t>
   </si>
   <si>
-    <t>La hoja es leida con exito y muestra mensaje de que los datos se encuentran completos</t>
+    <t>La hoja es leida con exito y muestra mensaje de que los datos se encuentran completos y muestra los datos que se encontraron, desde los headers hasta los datos en las siguientes filas</t>
   </si>
   <si>
     <t>Ausencia de todos los Encabezados</t>
@@ -345,10 +348,7 @@
     <t>El programa  revisar desde la primera fila que datos hacen falta, en este caso que hace falta indicar que los headers no  fuero encontrados y faltan</t>
   </si>
   <si>
-    <t>In progress</t>
-  </si>
-  <si>
-    <t>El programa indice cuando Falta solo una columa, e infdica el nombre, si faltan mas indica las que falten, si faltan todasde igual forma lo dice esto cuando analiza desde la A1 a lo que sigue</t>
+    <t>El programa lee el archivo y da mensaje de "Error critico hace falta los siguientes datos" y  muestra la lista de todos los datos que falta, en este caso muestra todos los headers</t>
   </si>
   <si>
     <t>Encabezados desordenados</t>
@@ -357,12 +357,15 @@
     <t>Los encabezados se encuentran completos pero en siferente orden a la lista definida</t>
   </si>
   <si>
-    <t>Los enccabezados se encuentran completos desde A1 sin embargo la lista primero se encuentra date lueco campaign etc, en este caso estos datos deben estar desordenados todos</t>
+    <t>Los enccabezados se encuentran completos desde A1 sin embargo la lista primero se encuentra date luego campaign etc, en este caso estos datos deben estar desordenados todos</t>
   </si>
   <si>
     <t>El programa debe ser capas de identificar que los datosse encuentran compeltosdesde la primera fila aunque estos se encuentren en desorden</t>
   </si>
   <si>
+    <t>El programa indica que los dtaos estan completos incluso cuando estan en desorden e imprime los headersy el contenido de la hoja</t>
+  </si>
+  <si>
     <t>Encabezados duplicados</t>
   </si>
   <si>
@@ -375,6 +378,9 @@
     <t>El programa debe ser capas de leer los datos e indicar que algunos estan duplicados e indicar cuales son para quese revise</t>
   </si>
   <si>
+    <t>El programa detecta las columas con datos duplicados e indica cuales son los que estan duplñiados para que se corrijan, en seguida termina</t>
+  </si>
+  <si>
     <t>Ausencia de algunos encabezados</t>
   </si>
   <si>
@@ -387,18 +393,72 @@
     <t>El programadebe ser capas de leer el archivo desde la celda A1, es decir primera fila del XLS e indicar cuales son los datos que faltan ya sea 1 o 2 datos como en ejemplo indicar que falta date, campaign e impressions</t>
   </si>
   <si>
+    <t>El programa detecta los encabezados que fueron ingresados y los compara correctamente indicando cuales son los que hace falta</t>
+  </si>
+  <si>
     <t>Desfase de Origen Vertical (Filas basura al inicio</t>
   </si>
   <si>
-    <t>Los encabezados reales comienzan en la columna 10. Las columnas 1 a 9 están vacías o contienen ruido. El script debe redefinir el origen dinámicamente.</t>
-  </si>
-  <si>
-    <t>La columna de informacion requerida comienza en la celda A10 y de la A1 a A9 no contiene informacion de ningun tipo, la columna de datos esta completa y en orden, no falta informacion, no tiene columnas extras ni datos duplicados, el desfase es unciamente vertical</t>
+    <t>Los encabezados reales comienzan en la celda A10. Las filas de la 1 a 9 están vacías o contienen ruido. El script debe redefinir el origen dinámicamente.</t>
+  </si>
+  <si>
+    <t>La fila de informacion requerida comienza en la celda A10 y de la A1 a A9 no contiene informacion de ningun tipo, la fila de datos esta completa y en orden, no falta informacion, no tiene columnas extras ni datos duplicados, el desfase es unciamente vertical</t>
   </si>
   <si>
     <t xml:space="preserve">El programa debe reajustar el header en cuanto encuentre la fila de datos requeridos, es decir si la informacion se encuentra en A10 comienza a analizar los headers,  como date,campaig, impression y al finalizar la comparacion de datos del archivo con los datos requeridos indicar que se encuentran completos </t>
   </si>
   <si>
+    <t>El programa detecta en donde se encuentran los encabezados en la nueva fila e imprime el analisis indicando que se encuentran completos</t>
+  </si>
+  <si>
+    <t>Desfase de Origen vertical con encabezados incompletos</t>
+  </si>
+  <si>
+    <t>Los encabezados reales comienzan en la celda A2. Las De la fila  A1 está vacía o contienen ruido. El script debe redefinir el origen dinámicamente e identificar que en esa nueva filase encuentra al menos el 50% de datos necesarios para comenzar con el analisis</t>
+  </si>
+  <si>
+    <t>La fila de informacion requerida comienza en la celda A2 y de la A1 no contiene informacion de ningun tipo, la fila de datos esta incompleta,  solo tiene  date, campaign, channel, impressions y total_click, es decir falta menos de la mitad de datos, no tiene columnas extras ni datos duplicados, el desfase es vertical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El programa debe reajustar el header en cuanto encuentre mas del  50% de coincidecia de datos en esa fila, es decir si  en la fila A2 detecta que al menos existen 5 de los encabezados comienza a analizar esa fila y su contenido y al finalizar la comparacion de datos del archivo con los datos requeridos indicar cuales hacen falta </t>
+  </si>
+  <si>
+    <t>El programa reajusta el headery analiza  ya que el archivo cumplio con mas del 50 pro no estaban completos indicaba cuales faltan</t>
+  </si>
+  <si>
+    <t>TC12B</t>
+  </si>
+  <si>
+    <t>Desfase de Origen vertical con mas de la mitad de encabezados incompletos</t>
+  </si>
+  <si>
+    <t>Los encabezados reales comienzan en la celda A6. Las De la fila  A1 a A5 están vacías o contienen ruido. El script debe redefinir el origen dinámicamente e identificar si en esa nueva filase se encuentra menos del 50% de datos necesarios para comenzar con el analisis</t>
+  </si>
+  <si>
+    <t>La fila de informacion requerida comienza en la celda A6 y de la A1 a A5 no contiene informacion de ningun tipo, la fila de datos esta incompleta,  solo tiene  date, campaign, channel e impressions es decir falta la mitad de datos o menos, no tiene columnas extras ni datos duplicados, el desfase es vertical</t>
+  </si>
+  <si>
+    <t>El programa debe reajustar el header si no encuentra al menos  50% de coincidecia de datos en alguna fila debe indicar que no se encuentra ninfuna fila con los datos necesarios e indicar que hacen falta todos los datos</t>
+  </si>
+  <si>
+    <t>El programa no encontro coincidencia en ninguna fila quecumpla el 50 por lo que indica que no encontro nada y se solicita revisar el archivo</t>
+  </si>
+  <si>
+    <t>TC12C</t>
+  </si>
+  <si>
+    <t>Desfase de Origen Vertical (Filas basura al inicio) y con header duplicados</t>
+  </si>
+  <si>
+    <t>Los encabezados reales comienzan en la celda A10. Las filas de la 1 a 9 están vacías o contienen ruido. El script debe redefinir el origen dinámicamente e identificar si estan duplicados los datos</t>
+  </si>
+  <si>
+    <t>Los encabezados reales comienzan en la celda A10. Las filas de la 1 a 9 están vacías o contienen ruido. El script debe redefinir el origen dinámicamente e identificar los datos que esten duplicados</t>
+  </si>
+  <si>
+    <t>El programa debe ser capaz de reajustar el nuevo header y analizar, si encuentra algun duplicados indicar que datos estan duplicados</t>
+  </si>
+  <si>
     <t>Desface der Columnas(Columnas basura al incio)</t>
   </si>
   <si>
@@ -409,6 +469,9 @@
   </si>
   <si>
     <t xml:space="preserve">El programa debe analizar desde la primer fila los datos , inidicar que se encuentran completos e imprimir los datos  filas y columnas encontradas, </t>
+  </si>
+  <si>
+    <t>Imprime los datosestan completos</t>
   </si>
   <si>
     <t>Desface de Columnas y Filas</t>
@@ -606,7 +669,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -676,6 +739,18 @@
     <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -683,9 +758,6 @@
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -795,6 +867,18 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing15.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
@@ -832,7 +916,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H29" displayName="Tabla_1" name="Tabla_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H32" displayName="Tabla_1" name="Tabla_1" id="1">
   <tableColumns count="8">
     <tableColumn name="-" id="1"/>
     <tableColumn name="Defecto a revisar" id="2"/>
@@ -1456,6 +1540,1529 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="D2" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="5">
+        <v>5168.0</v>
+      </c>
+      <c r="H2" s="5">
+        <v>134.0</v>
+      </c>
+      <c r="I2" s="5">
+        <v>258.0</v>
+      </c>
+      <c r="J2" s="4">
+        <v>362.0</v>
+      </c>
+      <c r="K2" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="D3" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="5">
+        <v>2314.0</v>
+      </c>
+      <c r="H3" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="I3" s="5">
+        <v>162.0</v>
+      </c>
+      <c r="J3" s="4">
+        <v>46.0</v>
+      </c>
+      <c r="K3" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="D4" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="5">
+        <v>3496.0</v>
+      </c>
+      <c r="H4" s="5">
+        <v>92.0</v>
+      </c>
+      <c r="I4" s="5">
+        <v>61.0</v>
+      </c>
+      <c r="J4" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="K4" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="D5" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="5">
+        <v>1790.0</v>
+      </c>
+      <c r="H5" s="5">
+        <v>87.0</v>
+      </c>
+      <c r="I5" s="5">
+        <v>370.0</v>
+      </c>
+      <c r="J5" s="4">
+        <v>54.0</v>
+      </c>
+      <c r="K5" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="D6" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="5">
+        <v>9764.0</v>
+      </c>
+      <c r="H6" s="5">
+        <v>53.0</v>
+      </c>
+      <c r="I6" s="5">
+        <v>118.0</v>
+      </c>
+      <c r="J6" s="4">
+        <v>293.0</v>
+      </c>
+      <c r="K6" s="6">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="D7" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="5">
+        <v>2912.0</v>
+      </c>
+      <c r="H7" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="I7" s="5">
+        <v>187.0</v>
+      </c>
+      <c r="J7" s="4">
+        <v>204.0</v>
+      </c>
+      <c r="K7" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="D8" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" s="5">
+        <v>4736.0</v>
+      </c>
+      <c r="H8" s="5">
+        <v>123.0</v>
+      </c>
+      <c r="I8" s="5">
+        <v>198.0</v>
+      </c>
+      <c r="J8" s="4">
+        <v>237.0</v>
+      </c>
+      <c r="K8" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="D9" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="5">
+        <v>7311.0</v>
+      </c>
+      <c r="H9" s="5">
+        <v>149.0</v>
+      </c>
+      <c r="I9" s="5">
+        <v>230.0</v>
+      </c>
+      <c r="J9" s="4">
+        <v>219.0</v>
+      </c>
+      <c r="K9" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="D10" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="5">
+        <v>4679.0</v>
+      </c>
+      <c r="H10" s="5">
+        <v>22.0</v>
+      </c>
+      <c r="I10" s="5">
+        <v>281.0</v>
+      </c>
+      <c r="J10" s="4">
+        <v>94.0</v>
+      </c>
+      <c r="K10" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="D11" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="5">
+        <v>4957.0</v>
+      </c>
+      <c r="H11" s="5">
+        <v>93.0</v>
+      </c>
+      <c r="I11" s="5">
+        <v>276.0</v>
+      </c>
+      <c r="J11" s="4">
+        <v>397.0</v>
+      </c>
+      <c r="K11" s="6">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="D12" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="5">
+        <v>2924.0</v>
+      </c>
+      <c r="H12" s="5">
+        <v>131.0</v>
+      </c>
+      <c r="I12" s="5">
+        <v>58.0</v>
+      </c>
+      <c r="J12" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="K12" s="6">
+        <v>7.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="D13" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="5">
+        <v>7200.0</v>
+      </c>
+      <c r="H13" s="5">
+        <v>96.0</v>
+      </c>
+      <c r="I13" s="5">
+        <v>315.0</v>
+      </c>
+      <c r="J13" s="6">
+        <v>288.0</v>
+      </c>
+      <c r="K13" s="6">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="D14" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="5">
+        <v>2177.0</v>
+      </c>
+      <c r="H14" s="5">
+        <v>23.0</v>
+      </c>
+      <c r="I14" s="5">
+        <v>262.0</v>
+      </c>
+      <c r="J14" s="6">
+        <v>131.0</v>
+      </c>
+      <c r="K14" s="6">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="D15" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="5">
+        <v>4367.0</v>
+      </c>
+      <c r="H15" s="5">
+        <v>126.0</v>
+      </c>
+      <c r="I15" s="5">
+        <v>161.0</v>
+      </c>
+      <c r="J15" s="6">
+        <v>262.0</v>
+      </c>
+      <c r="K15" s="6">
+        <v>6.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="11">
+      <c r="C11" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="C12" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F12" s="5">
+        <v>5168.0</v>
+      </c>
+      <c r="G12" s="5">
+        <v>134.0</v>
+      </c>
+      <c r="H12" s="5">
+        <v>258.0</v>
+      </c>
+      <c r="I12" s="4">
+        <v>362.0</v>
+      </c>
+      <c r="J12" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="5">
+        <v>2314.0</v>
+      </c>
+      <c r="G13" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="H13" s="5">
+        <v>162.0</v>
+      </c>
+      <c r="I13" s="4">
+        <v>46.0</v>
+      </c>
+      <c r="J13" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="5">
+        <v>3496.0</v>
+      </c>
+      <c r="G14" s="5">
+        <v>92.0</v>
+      </c>
+      <c r="H14" s="5">
+        <v>61.0</v>
+      </c>
+      <c r="I14" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="J14" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="5">
+        <v>1790.0</v>
+      </c>
+      <c r="G15" s="5">
+        <v>87.0</v>
+      </c>
+      <c r="H15" s="5">
+        <v>370.0</v>
+      </c>
+      <c r="I15" s="4">
+        <v>54.0</v>
+      </c>
+      <c r="J15" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="C16" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="5">
+        <v>9764.0</v>
+      </c>
+      <c r="G16" s="5">
+        <v>53.0</v>
+      </c>
+      <c r="H16" s="5">
+        <v>118.0</v>
+      </c>
+      <c r="I16" s="4">
+        <v>293.0</v>
+      </c>
+      <c r="J16" s="6">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="5">
+        <v>2912.0</v>
+      </c>
+      <c r="G17" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="H17" s="5">
+        <v>187.0</v>
+      </c>
+      <c r="I17" s="4">
+        <v>204.0</v>
+      </c>
+      <c r="J17" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="5">
+        <v>4736.0</v>
+      </c>
+      <c r="G18" s="5">
+        <v>123.0</v>
+      </c>
+      <c r="H18" s="5">
+        <v>198.0</v>
+      </c>
+      <c r="I18" s="4">
+        <v>237.0</v>
+      </c>
+      <c r="J18" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" s="5">
+        <v>7311.0</v>
+      </c>
+      <c r="G19" s="5">
+        <v>149.0</v>
+      </c>
+      <c r="H19" s="5">
+        <v>230.0</v>
+      </c>
+      <c r="I19" s="4">
+        <v>219.0</v>
+      </c>
+      <c r="J19" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="5">
+        <v>4679.0</v>
+      </c>
+      <c r="G20" s="5">
+        <v>22.0</v>
+      </c>
+      <c r="H20" s="5">
+        <v>281.0</v>
+      </c>
+      <c r="I20" s="4">
+        <v>94.0</v>
+      </c>
+      <c r="J20" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="5">
+        <v>4957.0</v>
+      </c>
+      <c r="G21" s="5">
+        <v>93.0</v>
+      </c>
+      <c r="H21" s="5">
+        <v>276.0</v>
+      </c>
+      <c r="I21" s="4">
+        <v>397.0</v>
+      </c>
+      <c r="J21" s="6">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="5">
+        <v>2924.0</v>
+      </c>
+      <c r="G22" s="5">
+        <v>131.0</v>
+      </c>
+      <c r="H22" s="5">
+        <v>58.0</v>
+      </c>
+      <c r="I22" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="J22" s="6">
+        <v>7.0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="C23" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F23" s="5">
+        <v>7200.0</v>
+      </c>
+      <c r="G23" s="5">
+        <v>96.0</v>
+      </c>
+      <c r="H23" s="5">
+        <v>315.0</v>
+      </c>
+      <c r="I23" s="6">
+        <v>288.0</v>
+      </c>
+      <c r="J23" s="6">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="5">
+        <v>2177.0</v>
+      </c>
+      <c r="G24" s="5">
+        <v>23.0</v>
+      </c>
+      <c r="H24" s="5">
+        <v>262.0</v>
+      </c>
+      <c r="I24" s="6">
+        <v>131.0</v>
+      </c>
+      <c r="J24" s="6">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25" s="5">
+        <v>4367.0</v>
+      </c>
+      <c r="G25" s="5">
+        <v>126.0</v>
+      </c>
+      <c r="H25" s="5">
+        <v>161.0</v>
+      </c>
+      <c r="I25" s="6">
+        <v>262.0</v>
+      </c>
+      <c r="J25" s="6">
+        <v>6.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="3" max="3" width="21.63"/>
+    <col customWidth="1" min="10" max="10" width="24.0"/>
+    <col customWidth="1" min="14" max="15" width="24.38"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="5">
+        <v>5168.0</v>
+      </c>
+      <c r="E2" s="5">
+        <v>134.0</v>
+      </c>
+      <c r="F2" s="5">
+        <v>258.0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>362.0</v>
+      </c>
+      <c r="H2" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="5">
+        <v>2314.0</v>
+      </c>
+      <c r="E3" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="F3" s="5">
+        <v>162.0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>46.0</v>
+      </c>
+      <c r="H3" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="5">
+        <v>3496.0</v>
+      </c>
+      <c r="E4" s="5">
+        <v>92.0</v>
+      </c>
+      <c r="F4" s="5">
+        <v>61.0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="H4" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="5">
+        <v>1790.0</v>
+      </c>
+      <c r="E5" s="5">
+        <v>87.0</v>
+      </c>
+      <c r="F5" s="5">
+        <v>370.0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>54.0</v>
+      </c>
+      <c r="H5" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="5">
+        <v>9764.0</v>
+      </c>
+      <c r="E6" s="5">
+        <v>53.0</v>
+      </c>
+      <c r="F6" s="5">
+        <v>118.0</v>
+      </c>
+      <c r="G6" s="4">
+        <v>293.0</v>
+      </c>
+      <c r="H6" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="5">
+        <v>2912.0</v>
+      </c>
+      <c r="E7" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="F7" s="5">
+        <v>187.0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>204.0</v>
+      </c>
+      <c r="H7" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="5">
+        <v>4736.0</v>
+      </c>
+      <c r="E8" s="5">
+        <v>123.0</v>
+      </c>
+      <c r="F8" s="5">
+        <v>198.0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>237.0</v>
+      </c>
+      <c r="H8" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="5">
+        <v>7311.0</v>
+      </c>
+      <c r="E9" s="5">
+        <v>149.0</v>
+      </c>
+      <c r="F9" s="5">
+        <v>230.0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>219.0</v>
+      </c>
+      <c r="H9" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="5">
+        <v>4679.0</v>
+      </c>
+      <c r="E10" s="5">
+        <v>22.0</v>
+      </c>
+      <c r="F10" s="5">
+        <v>281.0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>94.0</v>
+      </c>
+      <c r="H10" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="2"/>
+      <c r="P10" s="2"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="5">
+        <v>4957.0</v>
+      </c>
+      <c r="E11" s="5">
+        <v>93.0</v>
+      </c>
+      <c r="F11" s="5">
+        <v>276.0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>397.0</v>
+      </c>
+      <c r="H11" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L11" s="4"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="5"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="5">
+        <v>2924.0</v>
+      </c>
+      <c r="E12" s="5">
+        <v>131.0</v>
+      </c>
+      <c r="F12" s="5">
+        <v>58.0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="H12" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L12" s="4"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="5"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="5">
+        <v>7200.0</v>
+      </c>
+      <c r="E13" s="5">
+        <v>96.0</v>
+      </c>
+      <c r="F13" s="5">
+        <v>315.0</v>
+      </c>
+      <c r="G13" s="6">
+        <v>288.0</v>
+      </c>
+      <c r="H13" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K13" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L13" s="4"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="2"/>
+      <c r="P13" s="5"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="5">
+        <v>2177.0</v>
+      </c>
+      <c r="E14" s="5">
+        <v>23.0</v>
+      </c>
+      <c r="F14" s="5">
+        <v>262.0</v>
+      </c>
+      <c r="G14" s="6">
+        <v>131.0</v>
+      </c>
+      <c r="H14" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L14" s="4"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="2"/>
+      <c r="P14" s="5"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="5">
+        <v>4367.0</v>
+      </c>
+      <c r="E15" s="5">
+        <v>126.0</v>
+      </c>
+      <c r="F15" s="5">
+        <v>161.0</v>
+      </c>
+      <c r="G15" s="6">
+        <v>262.0</v>
+      </c>
+      <c r="H15" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L15" s="4"/>
+      <c r="M15" s="6"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="2"/>
+      <c r="P15" s="5"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="4"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="6"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="2"/>
+      <c r="P16" s="5"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="4"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="6"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="2"/>
+      <c r="P17" s="5"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="4"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
+      <c r="M18" s="6"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="2"/>
+      <c r="P18" s="5"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="4"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
+      <c r="M19" s="6"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="2"/>
+      <c r="P19" s="5"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="4"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="6"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="2"/>
+      <c r="P20" s="5"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="4"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="6"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="2"/>
+      <c r="P21" s="5"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="6"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="6"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="3"/>
+      <c r="P22" s="5"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="6"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="5"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="6"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="6"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="6"/>
+      <c r="N24" s="6"/>
+      <c r="O24" s="3"/>
+      <c r="P24" s="5"/>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="5" max="5" width="24.38"/>
     <col customWidth="1" min="6" max="6" width="16.88"/>
@@ -2067,7 +3674,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2481,7 +4088,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2715,12 +4322,12 @@
       <c r="E11" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="F11" s="15" t="s">
-        <v>107</v>
+      <c r="F11" s="13" t="s">
+        <v>77</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
@@ -2728,20 +4335,24 @@
         <v>47</v>
       </c>
       <c r="B12" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="D12" s="13" t="s">
         <v>110</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="E12" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="F12" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" s="21"/>
+      <c r="H12" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="F12" s="15"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="13" t="s">
@@ -2759,314 +4370,394 @@
       <c r="E13" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="F13" s="15"/>
+      <c r="F13" s="13" t="s">
+        <v>77</v>
+      </c>
       <c r="G13" s="21"/>
-      <c r="H13" s="21"/>
+      <c r="H13" s="13" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="13" t="s">
         <v>51</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="F14" s="15"/>
+        <v>121</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>77</v>
+      </c>
       <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
+      <c r="H14" s="13" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="13" t="s">
         <v>60</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="F15" s="15" t="s">
-        <v>107</v>
+        <v>126</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>77</v>
       </c>
       <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
+      <c r="H15" s="13" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="13" t="s">
         <v>62</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="F16" s="15" t="s">
-        <v>107</v>
+        <v>131</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>77</v>
       </c>
       <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
+      <c r="H16" s="13" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" s="22"/>
+      <c r="H17" s="13" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="18" ht="22.5" customHeight="1">
+      <c r="A18" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="F18" s="23"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="25"/>
+    </row>
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="A19" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="F17" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22"/>
-    </row>
-    <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="17" t="s">
+      <c r="B19" s="23" t="s">
+        <v>144</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>145</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="G19" s="24"/>
+      <c r="H19" s="25" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="C18" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="D18" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>136</v>
-      </c>
-      <c r="F18" s="17" t="s">
+      <c r="B20" s="23" t="s">
+        <v>149</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="F20" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-    </row>
-    <row r="19" ht="22.5" customHeight="1">
-      <c r="A19" s="17" t="s">
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+    </row>
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="B19" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="C19" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="D19" s="17" t="s">
-        <v>139</v>
-      </c>
-      <c r="E19" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="F19" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-    </row>
-    <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="23"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-    </row>
-    <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="23"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
+      <c r="B21" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="C21" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="D21" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="E21" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
     </row>
     <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="B22" s="23" t="s">
+        <v>157</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="E22" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="G22" s="26"/>
+      <c r="H22" s="26"/>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="27"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="27"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B25" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="C22" s="19" t="s">
+      <c r="C25" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="D22" s="19" t="s">
+      <c r="D25" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
-    </row>
-    <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B23" s="26" t="s">
-        <v>142</v>
-      </c>
-      <c r="C23" s="26" t="s">
-        <v>143</v>
-      </c>
-      <c r="D23" s="26" t="s">
-        <v>144</v>
-      </c>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-    </row>
-    <row r="24" ht="22.5" customHeight="1">
-      <c r="A24" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="B24" s="26" t="s">
-        <v>145</v>
-      </c>
-      <c r="C24" s="26" t="s">
-        <v>146</v>
-      </c>
-      <c r="D24" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="28"/>
-      <c r="H24" s="28"/>
-    </row>
-    <row r="25" ht="22.5" customHeight="1">
-      <c r="A25" s="25" t="s">
-        <v>56</v>
-      </c>
-      <c r="B25" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="C25" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="D25" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="E25" s="27"/>
-      <c r="F25" s="27"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
       <c r="G25" s="28"/>
       <c r="H25" s="28"/>
     </row>
     <row r="26" ht="22.5" customHeight="1">
-      <c r="A26" s="25" t="s">
-        <v>151</v>
-      </c>
-      <c r="B26" s="26" t="s">
-        <v>152</v>
-      </c>
-      <c r="C26" s="26" t="s">
-        <v>153</v>
-      </c>
-      <c r="D26" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="E26" s="27"/>
-      <c r="F26" s="27"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="28"/>
+      <c r="A26" s="29" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="C26" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="E26" s="30"/>
+      <c r="F26" s="30"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
     </row>
     <row r="27" ht="22.5" customHeight="1">
       <c r="A27" s="29" t="s">
-        <v>155</v>
-      </c>
-      <c r="B27" s="30" t="s">
-        <v>156</v>
-      </c>
-      <c r="C27" s="30" t="s">
-        <v>157</v>
-      </c>
-      <c r="D27" s="26" t="s">
-        <v>158</v>
-      </c>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="32"/>
+        <v>58</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="C27" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="31"/>
+      <c r="H27" s="31"/>
     </row>
     <row r="28" ht="22.5" customHeight="1">
-      <c r="A28" s="30" t="s">
-        <v>159</v>
-      </c>
-      <c r="B28" s="30" t="s">
-        <v>160</v>
-      </c>
-      <c r="C28" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="D28" s="26" t="s">
-        <v>162</v>
-      </c>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="32"/>
+      <c r="A28" s="29" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="C28" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="31"/>
     </row>
     <row r="29" ht="22.5" customHeight="1">
-      <c r="A29" s="23"/>
-      <c r="B29" s="23"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="33"/>
-    </row>
-    <row r="31">
-      <c r="C31" s="7"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="7"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="s">
-        <v>163</v>
-      </c>
-      <c r="B38" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>166</v>
+      <c r="A29" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="B29" s="23" t="s">
+        <v>172</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>174</v>
+      </c>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="31"/>
+    </row>
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="A30" s="32" t="s">
+        <v>175</v>
+      </c>
+      <c r="B30" s="33" t="s">
+        <v>176</v>
+      </c>
+      <c r="C30" s="33" t="s">
+        <v>177</v>
+      </c>
+      <c r="D30" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="E30" s="34"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="35"/>
+      <c r="H30" s="35"/>
+    </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="A31" s="33" t="s">
+        <v>179</v>
+      </c>
+      <c r="B31" s="33" t="s">
+        <v>180</v>
+      </c>
+      <c r="C31" s="33" t="s">
+        <v>181</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="E31" s="34"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="35"/>
+      <c r="H31" s="35"/>
+    </row>
+    <row r="32" ht="22.5" customHeight="1">
+      <c r="A32" s="27"/>
+      <c r="B32" s="27"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="36"/>
+      <c r="H32" s="36"/>
+    </row>
+    <row r="34">
+      <c r="C34" s="7"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="7"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -5297,394 +6988,259 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
-    <row r="1">
-      <c r="D1" s="1" t="s">
+    <row r="2">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="D2" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="2" t="s">
+    </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="5">
+      <c r="D3" s="5">
         <v>5168.0</v>
       </c>
-      <c r="H2" s="5">
+      <c r="E3" s="5">
         <v>134.0</v>
       </c>
-      <c r="I2" s="5">
-        <v>258.0</v>
-      </c>
-      <c r="J2" s="4">
-        <v>362.0</v>
-      </c>
-      <c r="K2" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="D3" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="2" t="s">
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="5">
+      <c r="D4" s="5">
         <v>2314.0</v>
       </c>
-      <c r="H3" s="5">
+      <c r="E4" s="5">
         <v>26.0</v>
       </c>
-      <c r="I3" s="5">
-        <v>162.0</v>
-      </c>
-      <c r="J3" s="4">
-        <v>46.0</v>
-      </c>
-      <c r="K3" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="D4" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="2" t="s">
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="5">
+      <c r="D5" s="5">
         <v>3496.0</v>
       </c>
-      <c r="H4" s="5">
+      <c r="E5" s="5">
         <v>92.0</v>
       </c>
-      <c r="I4" s="5">
-        <v>61.0</v>
-      </c>
-      <c r="J4" s="4">
-        <v>175.0</v>
-      </c>
-      <c r="K4" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="D5" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="2" t="s">
+    </row>
+    <row r="6">
+      <c r="A6" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="5">
+      <c r="D6" s="5">
         <v>1790.0</v>
       </c>
-      <c r="H5" s="5">
+      <c r="E6" s="5">
         <v>87.0</v>
       </c>
-      <c r="I5" s="5">
-        <v>370.0</v>
-      </c>
-      <c r="J5" s="4">
-        <v>54.0</v>
-      </c>
-      <c r="K5" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="D6" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="2" t="s">
+    </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="5">
+      <c r="D7" s="5">
         <v>9764.0</v>
       </c>
-      <c r="H6" s="5">
+      <c r="E7" s="5">
         <v>53.0</v>
       </c>
-      <c r="I6" s="5">
-        <v>118.0</v>
-      </c>
-      <c r="J6" s="4">
-        <v>293.0</v>
-      </c>
-      <c r="K6" s="6">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="D7" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" s="2" t="s">
+    </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="5">
+      <c r="D8" s="5">
         <v>2912.0</v>
       </c>
-      <c r="H7" s="5">
+      <c r="E8" s="5">
         <v>26.0</v>
       </c>
-      <c r="I7" s="5">
-        <v>187.0</v>
-      </c>
-      <c r="J7" s="4">
-        <v>204.0</v>
-      </c>
-      <c r="K7" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="D8" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="2" t="s">
+    </row>
+    <row r="9">
+      <c r="A9" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="5">
+      <c r="D9" s="5">
         <v>4736.0</v>
       </c>
-      <c r="H8" s="5">
+      <c r="E9" s="5">
         <v>123.0</v>
       </c>
-      <c r="I8" s="5">
-        <v>198.0</v>
-      </c>
-      <c r="J8" s="4">
-        <v>237.0</v>
-      </c>
-      <c r="K8" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="D9" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="2" t="s">
+    </row>
+    <row r="10">
+      <c r="A10" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="5">
+      <c r="D10" s="5">
         <v>7311.0</v>
       </c>
-      <c r="H9" s="5">
+      <c r="E10" s="5">
         <v>149.0</v>
       </c>
-      <c r="I9" s="5">
-        <v>230.0</v>
-      </c>
-      <c r="J9" s="4">
-        <v>219.0</v>
-      </c>
-      <c r="K9" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="D10" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="2" t="s">
+    </row>
+    <row r="11">
+      <c r="A11" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="5">
+      <c r="D11" s="5">
         <v>4679.0</v>
       </c>
-      <c r="H10" s="5">
+      <c r="E11" s="5">
         <v>22.0</v>
       </c>
-      <c r="I10" s="5">
-        <v>281.0</v>
-      </c>
-      <c r="J10" s="4">
-        <v>94.0</v>
-      </c>
-      <c r="K10" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="D11" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F11" s="2" t="s">
+    </row>
+    <row r="12">
+      <c r="A12" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G11" s="5">
+      <c r="D12" s="5">
         <v>4957.0</v>
       </c>
-      <c r="H11" s="5">
+      <c r="E12" s="5">
         <v>93.0</v>
       </c>
-      <c r="I11" s="5">
-        <v>276.0</v>
-      </c>
-      <c r="J11" s="4">
-        <v>397.0</v>
-      </c>
-      <c r="K11" s="6">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="D12" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F12" s="2" t="s">
+    </row>
+    <row r="13">
+      <c r="A13" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G12" s="5">
+      <c r="D13" s="5">
         <v>2924.0</v>
       </c>
-      <c r="H12" s="5">
+      <c r="E13" s="5">
         <v>131.0</v>
       </c>
-      <c r="I12" s="5">
-        <v>58.0</v>
-      </c>
-      <c r="J12" s="4">
-        <v>175.0</v>
-      </c>
-      <c r="K12" s="6">
-        <v>7.0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="D13" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F13" s="3" t="s">
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G13" s="5">
+      <c r="D14" s="5">
         <v>7200.0</v>
       </c>
-      <c r="H13" s="5">
+      <c r="E14" s="5">
         <v>96.0</v>
       </c>
-      <c r="I13" s="5">
-        <v>315.0</v>
-      </c>
-      <c r="J13" s="6">
-        <v>288.0</v>
-      </c>
-      <c r="K13" s="6">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="D14" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F14" s="3" t="s">
+    </row>
+    <row r="15">
+      <c r="A15" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G14" s="5">
+      <c r="D15" s="5">
         <v>2177.0</v>
       </c>
-      <c r="H14" s="5">
+      <c r="E15" s="5">
         <v>23.0</v>
       </c>
-      <c r="I14" s="5">
-        <v>262.0</v>
-      </c>
-      <c r="J14" s="6">
-        <v>131.0</v>
-      </c>
-      <c r="K14" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="D15" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F15" s="3" t="s">
+    </row>
+    <row r="16">
+      <c r="A16" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G15" s="5">
+      <c r="D16" s="5">
         <v>4367.0</v>
       </c>
-      <c r="H15" s="5">
+      <c r="E16" s="5">
         <v>126.0</v>
-      </c>
-      <c r="I15" s="5">
-        <v>161.0</v>
-      </c>
-      <c r="J15" s="6">
-        <v>262.0</v>
-      </c>
-      <c r="K15" s="6">
-        <v>6.0</v>
       </c>
     </row>
   </sheetData>
@@ -5699,395 +7255,230 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
+    <row r="6">
+      <c r="A6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="2"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="5">
+        <v>5168.0</v>
+      </c>
+      <c r="E7" s="5"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="5">
+        <v>2314.0</v>
+      </c>
+      <c r="E8" s="5"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="5">
+        <v>3496.0</v>
+      </c>
+      <c r="E9" s="5"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="5">
+        <v>1790.0</v>
+      </c>
+      <c r="E10" s="5"/>
+    </row>
     <row r="11">
-      <c r="C11" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="A11" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="5">
+        <v>9764.0</v>
+      </c>
+      <c r="E11" s="5"/>
     </row>
     <row r="12">
-      <c r="C12" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="2" t="s">
+      <c r="A12" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="5">
+        <v>2912.0</v>
+      </c>
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="5">
+        <v>4736.0</v>
+      </c>
+      <c r="E13" s="5"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F12" s="5">
-        <v>5168.0</v>
-      </c>
-      <c r="G12" s="5">
-        <v>134.0</v>
-      </c>
-      <c r="H12" s="5">
-        <v>258.0</v>
-      </c>
-      <c r="I12" s="4">
-        <v>362.0</v>
-      </c>
-      <c r="J12" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="C13" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="D14" s="5">
+        <v>7311.0</v>
+      </c>
+      <c r="E14" s="5"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="5">
-        <v>2314.0</v>
-      </c>
-      <c r="G13" s="5">
-        <v>26.0</v>
-      </c>
-      <c r="H13" s="5">
-        <v>162.0</v>
-      </c>
-      <c r="I13" s="4">
-        <v>46.0</v>
-      </c>
-      <c r="J13" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="C14" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="D15" s="5">
+        <v>4679.0</v>
+      </c>
+      <c r="E15" s="5"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F14" s="5">
-        <v>3496.0</v>
-      </c>
-      <c r="G14" s="5">
-        <v>92.0</v>
-      </c>
-      <c r="H14" s="5">
-        <v>61.0</v>
-      </c>
-      <c r="I14" s="4">
-        <v>175.0</v>
-      </c>
-      <c r="J14" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="C15" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="2" t="s">
+      <c r="D16" s="5">
+        <v>4957.0</v>
+      </c>
+      <c r="E16" s="5"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="5">
-        <v>1790.0</v>
-      </c>
-      <c r="G15" s="5">
-        <v>87.0</v>
-      </c>
-      <c r="H15" s="5">
-        <v>370.0</v>
-      </c>
-      <c r="I15" s="4">
-        <v>54.0</v>
-      </c>
-      <c r="J15" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="C16" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" s="2" t="s">
+      <c r="D17" s="5">
+        <v>2924.0</v>
+      </c>
+      <c r="E17" s="5"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F16" s="5">
-        <v>9764.0</v>
-      </c>
-      <c r="G16" s="5">
-        <v>53.0</v>
-      </c>
-      <c r="H16" s="5">
-        <v>118.0</v>
-      </c>
-      <c r="I16" s="4">
-        <v>293.0</v>
-      </c>
-      <c r="J16" s="6">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="C17" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E17" s="2" t="s">
+      <c r="D18" s="5">
+        <v>7200.0</v>
+      </c>
+      <c r="E18" s="5"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F17" s="5">
-        <v>2912.0</v>
-      </c>
-      <c r="G17" s="5">
-        <v>26.0</v>
-      </c>
-      <c r="H17" s="5">
-        <v>187.0</v>
-      </c>
-      <c r="I17" s="4">
-        <v>204.0</v>
-      </c>
-      <c r="J17" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="C18" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E18" s="2" t="s">
+      <c r="D19" s="5">
+        <v>2177.0</v>
+      </c>
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F18" s="5">
-        <v>4736.0</v>
-      </c>
-      <c r="G18" s="5">
-        <v>123.0</v>
-      </c>
-      <c r="H18" s="5">
-        <v>198.0</v>
-      </c>
-      <c r="I18" s="4">
-        <v>237.0</v>
-      </c>
-      <c r="J18" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="C19" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F19" s="5">
-        <v>7311.0</v>
-      </c>
-      <c r="G19" s="5">
-        <v>149.0</v>
-      </c>
-      <c r="H19" s="5">
-        <v>230.0</v>
-      </c>
-      <c r="I19" s="4">
-        <v>219.0</v>
-      </c>
-      <c r="J19" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="C20" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F20" s="5">
-        <v>4679.0</v>
-      </c>
-      <c r="G20" s="5">
-        <v>22.0</v>
-      </c>
-      <c r="H20" s="5">
-        <v>281.0</v>
-      </c>
-      <c r="I20" s="4">
-        <v>94.0</v>
-      </c>
-      <c r="J20" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="C21" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F21" s="5">
-        <v>4957.0</v>
-      </c>
-      <c r="G21" s="5">
-        <v>93.0</v>
-      </c>
-      <c r="H21" s="5">
-        <v>276.0</v>
-      </c>
-      <c r="I21" s="4">
-        <v>397.0</v>
-      </c>
-      <c r="J21" s="6">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="C22" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F22" s="5">
-        <v>2924.0</v>
-      </c>
-      <c r="G22" s="5">
-        <v>131.0</v>
-      </c>
-      <c r="H22" s="5">
-        <v>58.0</v>
-      </c>
-      <c r="I22" s="4">
-        <v>175.0</v>
-      </c>
-      <c r="J22" s="6">
-        <v>7.0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="C23" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F23" s="5">
-        <v>7200.0</v>
-      </c>
-      <c r="G23" s="5">
-        <v>96.0</v>
-      </c>
-      <c r="H23" s="5">
-        <v>315.0</v>
-      </c>
-      <c r="I23" s="6">
-        <v>288.0</v>
-      </c>
-      <c r="J23" s="6">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="C24" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F24" s="5">
-        <v>2177.0</v>
-      </c>
-      <c r="G24" s="5">
-        <v>23.0</v>
-      </c>
-      <c r="H24" s="5">
-        <v>262.0</v>
-      </c>
-      <c r="I24" s="6">
-        <v>131.0</v>
-      </c>
-      <c r="J24" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="C25" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F25" s="5">
+      <c r="D20" s="5">
         <v>4367.0</v>
       </c>
-      <c r="G25" s="5">
-        <v>126.0</v>
-      </c>
-      <c r="H25" s="5">
-        <v>161.0</v>
-      </c>
-      <c r="I25" s="6">
-        <v>262.0</v>
-      </c>
-      <c r="J25" s="6">
-        <v>6.0</v>
-      </c>
+      <c r="E20" s="5"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -6101,712 +7492,488 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="3" max="3" width="21.63"/>
-    <col customWidth="1" min="10" max="10" width="24.0"/>
-    <col customWidth="1" min="14" max="15" width="24.38"/>
+    <col customWidth="1" min="10" max="10" width="24.38"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="11">
+      <c r="A11" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="L1" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="5">
-        <v>5168.0</v>
-      </c>
-      <c r="E2" s="5">
-        <v>134.0</v>
-      </c>
-      <c r="F2" s="5">
-        <v>258.0</v>
-      </c>
-      <c r="G2" s="4">
-        <v>362.0</v>
-      </c>
-      <c r="H2" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="5">
-        <v>2314.0</v>
-      </c>
-      <c r="E3" s="5">
-        <v>26.0</v>
-      </c>
-      <c r="F3" s="5">
-        <v>162.0</v>
-      </c>
-      <c r="G3" s="4">
-        <v>46.0</v>
-      </c>
-      <c r="H3" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="5">
-        <v>3496.0</v>
-      </c>
-      <c r="E4" s="5">
-        <v>92.0</v>
-      </c>
-      <c r="F4" s="5">
-        <v>61.0</v>
-      </c>
-      <c r="G4" s="4">
-        <v>175.0</v>
-      </c>
-      <c r="H4" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="5">
-        <v>1790.0</v>
-      </c>
-      <c r="E5" s="5">
-        <v>87.0</v>
-      </c>
-      <c r="F5" s="5">
-        <v>370.0</v>
-      </c>
-      <c r="G5" s="4">
-        <v>54.0</v>
-      </c>
-      <c r="H5" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="5">
-        <v>9764.0</v>
-      </c>
-      <c r="E6" s="5">
-        <v>53.0</v>
-      </c>
-      <c r="F6" s="5">
-        <v>118.0</v>
-      </c>
-      <c r="G6" s="4">
-        <v>293.0</v>
-      </c>
-      <c r="H6" s="6">
-        <v>3.0</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K6" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="5">
-        <v>2912.0</v>
-      </c>
-      <c r="E7" s="5">
-        <v>26.0</v>
-      </c>
-      <c r="F7" s="5">
-        <v>187.0</v>
-      </c>
-      <c r="G7" s="4">
-        <v>204.0</v>
-      </c>
-      <c r="H7" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="5">
-        <v>4736.0</v>
-      </c>
-      <c r="E8" s="5">
-        <v>123.0</v>
-      </c>
-      <c r="F8" s="5">
-        <v>198.0</v>
-      </c>
-      <c r="G8" s="4">
-        <v>237.0</v>
-      </c>
-      <c r="H8" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="5">
-        <v>7311.0</v>
-      </c>
-      <c r="E9" s="5">
-        <v>149.0</v>
-      </c>
-      <c r="F9" s="5">
-        <v>230.0</v>
-      </c>
-      <c r="G9" s="4">
-        <v>219.0</v>
-      </c>
-      <c r="H9" s="6">
-        <v>4.0</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J9" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="5">
-        <v>4679.0</v>
-      </c>
-      <c r="E10" s="5">
-        <v>22.0</v>
-      </c>
-      <c r="F10" s="5">
-        <v>281.0</v>
-      </c>
-      <c r="G10" s="4">
-        <v>94.0</v>
-      </c>
-      <c r="H10" s="6">
-        <v>1.0</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="5">
-        <v>4957.0</v>
-      </c>
-      <c r="E11" s="5">
-        <v>93.0</v>
-      </c>
-      <c r="F11" s="5">
-        <v>276.0</v>
-      </c>
-      <c r="G11" s="4">
-        <v>397.0</v>
-      </c>
-      <c r="H11" s="6">
-        <v>5.0</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K11" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="L11" s="4"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="4"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="5"/>
+      <c r="I11" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4">
         <v>45658.0</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D12" s="5">
-        <v>2924.0</v>
+        <v>5168.0</v>
       </c>
       <c r="E12" s="5">
-        <v>131.0</v>
+        <v>134.0</v>
       </c>
       <c r="F12" s="5">
-        <v>58.0</v>
+        <v>258.0</v>
       </c>
       <c r="G12" s="4">
-        <v>175.0</v>
+        <v>362.0</v>
       </c>
       <c r="H12" s="6">
-        <v>7.0</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J12" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K12" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="L12" s="4"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="2"/>
-      <c r="P12" s="5"/>
+        <v>4.0</v>
+      </c>
+      <c r="I12" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4">
         <v>45658.0</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>13</v>
+      <c r="B13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="D13" s="5">
-        <v>7200.0</v>
+        <v>2314.0</v>
       </c>
       <c r="E13" s="5">
-        <v>96.0</v>
+        <v>26.0</v>
       </c>
       <c r="F13" s="5">
-        <v>315.0</v>
-      </c>
-      <c r="G13" s="6">
-        <v>288.0</v>
+        <v>162.0</v>
+      </c>
+      <c r="G13" s="4">
+        <v>46.0</v>
       </c>
       <c r="H13" s="6">
-        <v>2.0</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K13" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="L13" s="4"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="4"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="5"/>
+        <v>1.0</v>
+      </c>
+      <c r="I13" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4">
         <v>45658.0</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>14</v>
+      <c r="B14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>11</v>
       </c>
       <c r="D14" s="5">
-        <v>2177.0</v>
+        <v>3496.0</v>
       </c>
       <c r="E14" s="5">
-        <v>23.0</v>
+        <v>92.0</v>
       </c>
       <c r="F14" s="5">
-        <v>262.0</v>
-      </c>
-      <c r="G14" s="6">
-        <v>131.0</v>
+        <v>61.0</v>
+      </c>
+      <c r="G14" s="4">
+        <v>175.0</v>
       </c>
       <c r="H14" s="6">
-        <v>0.0</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J14" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K14" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="L14" s="4"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="5"/>
+        <v>1.0</v>
+      </c>
+      <c r="I14" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4">
         <v>45658.0</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="3" t="s">
+      <c r="B15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="5">
+        <v>1790.0</v>
+      </c>
+      <c r="E15" s="5">
+        <v>87.0</v>
+      </c>
+      <c r="F15" s="5">
+        <v>370.0</v>
+      </c>
+      <c r="G15" s="4">
+        <v>54.0</v>
+      </c>
+      <c r="H15" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="I15" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="5">
+        <v>9764.0</v>
+      </c>
+      <c r="E16" s="5">
+        <v>53.0</v>
+      </c>
+      <c r="F16" s="5">
+        <v>118.0</v>
+      </c>
+      <c r="G16" s="4">
+        <v>293.0</v>
+      </c>
+      <c r="H16" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="I16" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="5">
+        <v>2912.0</v>
+      </c>
+      <c r="E17" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="F17" s="5">
+        <v>187.0</v>
+      </c>
+      <c r="G17" s="4">
+        <v>204.0</v>
+      </c>
+      <c r="H17" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="I17" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D18" s="5">
+        <v>4736.0</v>
+      </c>
+      <c r="E18" s="5">
+        <v>123.0</v>
+      </c>
+      <c r="F18" s="5">
+        <v>198.0</v>
+      </c>
+      <c r="G18" s="4">
+        <v>237.0</v>
+      </c>
+      <c r="H18" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="I18" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="5">
+        <v>7311.0</v>
+      </c>
+      <c r="E19" s="5">
+        <v>149.0</v>
+      </c>
+      <c r="F19" s="5">
+        <v>230.0</v>
+      </c>
+      <c r="G19" s="4">
+        <v>219.0</v>
+      </c>
+      <c r="H19" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="I19" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="5">
+        <v>4679.0</v>
+      </c>
+      <c r="E20" s="5">
+        <v>22.0</v>
+      </c>
+      <c r="F20" s="5">
+        <v>281.0</v>
+      </c>
+      <c r="G20" s="4">
+        <v>94.0</v>
+      </c>
+      <c r="H20" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="I20" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="5">
+        <v>4957.0</v>
+      </c>
+      <c r="E21" s="5">
+        <v>93.0</v>
+      </c>
+      <c r="F21" s="5">
+        <v>276.0</v>
+      </c>
+      <c r="G21" s="4">
+        <v>397.0</v>
+      </c>
+      <c r="H21" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="I21" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="5">
+        <v>2924.0</v>
+      </c>
+      <c r="E22" s="5">
+        <v>131.0</v>
+      </c>
+      <c r="F22" s="5">
+        <v>58.0</v>
+      </c>
+      <c r="G22" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="H22" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="I22" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="5">
+        <v>7200.0</v>
+      </c>
+      <c r="E23" s="5">
+        <v>96.0</v>
+      </c>
+      <c r="F23" s="5">
+        <v>315.0</v>
+      </c>
+      <c r="G23" s="6">
+        <v>288.0</v>
+      </c>
+      <c r="H23" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="I23" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="5">
+        <v>2177.0</v>
+      </c>
+      <c r="E24" s="5">
+        <v>23.0</v>
+      </c>
+      <c r="F24" s="5">
+        <v>262.0</v>
+      </c>
+      <c r="G24" s="6">
+        <v>131.0</v>
+      </c>
+      <c r="H24" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="I24" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="5">
         <v>4367.0</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E25" s="5">
         <v>126.0</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F25" s="5">
         <v>161.0</v>
       </c>
-      <c r="G15" s="6">
+      <c r="G25" s="6">
         <v>262.0</v>
       </c>
-      <c r="H15" s="6">
+      <c r="H25" s="6">
         <v>6.0</v>
       </c>
-      <c r="I15" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="J15" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K15" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="L15" s="4"/>
-      <c r="M15" s="6"/>
-      <c r="N15" s="4"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="5"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="4"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="6"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="5"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="4"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="6"/>
-      <c r="N17" s="4"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="5"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="4"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="6"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="2"/>
-      <c r="P18" s="5"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="4"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="6"/>
-      <c r="N19" s="4"/>
-      <c r="O19" s="2"/>
-      <c r="P19" s="5"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="4"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
-      <c r="M20" s="6"/>
-      <c r="N20" s="4"/>
-      <c r="O20" s="2"/>
-      <c r="P20" s="5"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="4"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
-      <c r="M21" s="6"/>
-      <c r="N21" s="4"/>
-      <c r="O21" s="2"/>
-      <c r="P21" s="5"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="6"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="6"/>
-      <c r="L22" s="4"/>
-      <c r="M22" s="6"/>
-      <c r="N22" s="6"/>
-      <c r="O22" s="3"/>
-      <c r="P22" s="5"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="6"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="6"/>
-      <c r="L23" s="4"/>
-      <c r="M23" s="6"/>
-      <c r="N23" s="6"/>
-      <c r="O23" s="3"/>
-      <c r="P23" s="5"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="6"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="6"/>
-      <c r="L24" s="4"/>
-      <c r="M24" s="6"/>
-      <c r="N24" s="6"/>
-      <c r="O24" s="3"/>
-      <c r="P24" s="5"/>
+      <c r="I25" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
cleanup: remove dead commented code (legacy .columns check); validate TC17-TC19; add TC13A and TC20; document results and Phase 2 (TC21-TC26)
</commit_message>
<xml_diff>
--- a/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
+++ b/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
@@ -17,9 +17,10 @@
     <sheet state="visible" name="TC16" sheetId="12" r:id="rId16"/>
     <sheet state="visible" name="TC17" sheetId="13" r:id="rId17"/>
     <sheet state="visible" name="TC18" sheetId="14" r:id="rId18"/>
-    <sheet state="visible" name="tc19" sheetId="15" r:id="rId19"/>
-    <sheet state="visible" name="Estructura logica" sheetId="16" r:id="rId20"/>
-    <sheet state="visible" name="TC Codigo" sheetId="17" r:id="rId21"/>
+    <sheet state="visible" name="TC19" sheetId="15" r:id="rId19"/>
+    <sheet state="visible" name="TC20" sheetId="16" r:id="rId20"/>
+    <sheet state="visible" name="Estructura logica" sheetId="17" r:id="rId21"/>
+    <sheet state="visible" name="TC Codigo" sheetId="18" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="218">
   <si>
     <t>date</t>
   </si>
@@ -266,9 +267,6 @@
     <t>Actual Result</t>
   </si>
   <si>
-    <t>Columna 1</t>
-  </si>
-  <si>
     <t>Excepción por Archivo Inexistente</t>
   </si>
   <si>
@@ -359,7 +357,7 @@
     <t xml:space="preserve">El programa debe indicar que los header se encuentran completos </t>
   </si>
   <si>
-    <t>La hoja es leida con exito y muestra mensaje de que los datos se encuentran completos y muestra los datos que se encontraron, desde los headers hasta los datos en las siguientes filas</t>
+    <t>El programa lee la hoja e indica de momento que se encontro el encabezado, la posicion de fila de encabezado, la coincidencia maxima, muestra la lista de entrada de datos, como no tiene datos adicionales muestra la traslitsh como vacia</t>
   </si>
   <si>
     <t>Ausencia de todos los Encabezados</t>
@@ -374,7 +372,7 @@
     <t>El programa de recorrer las nrows y si no encuentra coincidencia indica que no encontro nada e indicar que hacel falta los headers</t>
   </si>
   <si>
-    <t>El programa lee el archivo y da mensaje de "Error critico hace falta los siguientes datos" y  muestra la lista de todos los datos que falta, en este caso muestra todos los headers</t>
+    <t>El programa recorre la la hoja y al no encontrar header de coincidencia indica que no fue encontrado y termina el programa, ya que no hay que evaluar no muestra trash data ni coincidencia, unicamente termina el programa al no encontrar coincidencia de ningun tipo a evaluar</t>
   </si>
   <si>
     <t>Encabezados desordenados</t>
@@ -389,7 +387,7 @@
     <t xml:space="preserve">El programa debe ser capas de identificar que los datos se encuentran compeltosdesde la primera fila aunque estos se encuentren en desorden, e indicar que no tiene columnas adicionales </t>
   </si>
   <si>
-    <t>El programa indica que los dtaos estan completos incluso cuando estan en desorden e imprime los headersy el contenido de la hoja</t>
+    <t>El programa lee el archivo y muestra la lista en orden que entra en el excel, es decir con desorden, esa fila de datos es evaluada, indica que no tiene trash data, duplicados falso y max coincidencia de 100</t>
   </si>
   <si>
     <t>Encabezados duplicados</t>
@@ -404,10 +402,7 @@
     <t xml:space="preserve">El programa debe ser capas de detectar los headers e indicar cuales estan duplicados y completos, que revise cuales son los correctos, adicional a ello mostrar un mensaje de que no tiene columnas extras </t>
   </si>
   <si>
-    <t>El programa detecta las columas con datos duplicados e indica cuales son los que estan duplñiados para que se corrijan, en seguida termina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pending </t>
+    <t>El programa encuentra una fila con max coincidencia, la evalua, indica los datos que se encuentran duplicados respecto a los datos que se requieren, es decir indica si date o un dato de la lista esta duplicado, la trash list esta vacia, duplicados true, completos true</t>
   </si>
   <si>
     <t>Ausencia de algunos encabezados</t>
@@ -422,7 +417,10 @@
     <t>El programadebe ser capas de leer el archivo desde la celda A1, es decir primera fila del XLS e indicar cuales son los datos que faltan ya sea 1 o 2 datos como en ejemplo indicar que falta date, campaign e impressions, y debe indicar que no hay columnas extras ni datos duplicados</t>
   </si>
   <si>
-    <t>El programa detecta los encabezados que fueron ingresados y los compara correctamente indicando cuales son los que hace falta</t>
+    <t xml:space="preserve">Pass </t>
+  </si>
+  <si>
+    <t>El programa recorre bien la fila, indica la max coincidencia encontrada, indica los datos que faltan, ya que hay columnas sin titulo la muestra como valores nan la cual se va a la lista de trash data, indica que no tiene duplicados</t>
   </si>
   <si>
     <t>Desface der Columnas(Columnas basura al incio)</t>
@@ -437,7 +435,7 @@
     <t>El programa debe analizar desde la primer fila los datos , inidicar que se encuentran completos e imprimir los datos  filas y columnas encontradas, indicar que no hay columnas extras y no hay datos duplicados</t>
   </si>
   <si>
-    <t>El programa indica cuales son los headers y al analizarlo indica que los datos estan completos</t>
+    <t>El programa indica la posicion del header, la max coincidencia, los primero valores se identifican como nan, los cuales se van a trash data, lo cual ahora e stru, en cuanto a duplicados indica que no se encuentran valores duplicados</t>
   </si>
   <si>
     <t>Encabezados duplicados y faltantes</t>
@@ -452,6 +450,9 @@
     <t>El programa debe decirle que tiene encabezados dupliados y mencionar que headers hacen falta, adicional indicar que no tiene columnas adicionales a los duplicados</t>
   </si>
   <si>
+    <t>El programa indica la posicion donde se encuentra el header, la lista de datos de entrada es evaluada, indica la max coincidencia encontrada, en valor de duplicados es true indica los valores duplicados y la trash data se encuentra vacia</t>
+  </si>
+  <si>
     <t>Columnas de comentarios adicionales</t>
   </si>
   <si>
@@ -464,7 +465,22 @@
     <t>El programa debe eliminar esa columna adicional ya que no es necesaria antes de procesar la informacion y debe mostrarle indicarle al usuario que columnas estan adicionales que no seran consideradas</t>
   </si>
   <si>
-    <t>In progress by refactor</t>
+    <t>El programa localiza bien la fila de max coincidencia, indica que headers fueron encontrados, y antes de contar valores duplicados saca los trash data que fueron encontrados en esa fila</t>
+  </si>
+  <si>
+    <t>TC13A</t>
+  </si>
+  <si>
+    <t>Valores duplicados y columnas adicionales, con headers faltantes y duplicados</t>
+  </si>
+  <si>
+    <t>El header se encuentra en la primera fila, con datos desordenados, faltan datos de los headers,  y se encuentran columnas de comentarios adicionales</t>
+  </si>
+  <si>
+    <t>El programa localiza la fila, identifica los datos de header que se encuentran duplicados, indica las filas que se encuentran de datos adicionales</t>
+  </si>
+  <si>
+    <t>El programa localiza la max coincidencia, indica que valores se encuentran duplicados, indica que valores se encuentra como trash que no son parte de los headers e indica cuales son los que faltan</t>
   </si>
   <si>
     <t>Desfase de forma horizontal con intercalado entre columas, datos duplicados, faltantes y comentarios adicionales</t>
@@ -479,6 +495,9 @@
     <t xml:space="preserve">El codigo debe de leer la fila correcta indicando que datos se encuentran duplicados y que datos faltan si es necesario para solicitar al usuario que lo corrija e indicar que columnas adicionales tiene y que estas no seran consideradas </t>
   </si>
   <si>
+    <t>El progrma a puede identioficar la fila de datos, muestra valores nan y valores de datos adicionales identificados como trash data, los limpia e indica cuales son los que faltan y los que se encuentran duplicados</t>
+  </si>
+  <si>
     <t>Desfase de Origen Vertical (Filas basura al inicio</t>
   </si>
   <si>
@@ -491,10 +510,7 @@
     <t>El programa debe reajustar el header en cuanto encuentre la fila de datos requeridos, es decir si la informacion se encuentra en A10 comienza a analizar los headers,  como date,campaig, impression y al finalizar la comparacion de datos del archivo con los datos requeridos indicar que se encuentran completos, que no tiene duplicados y no hay comentarios adicionales</t>
   </si>
   <si>
-    <t>Pendieng evaluation by refactor</t>
-  </si>
-  <si>
-    <t>El programa detecta en donde se encuentran los encabezados en la nueva fila e imprime el analisis indicando que se encuentran completos</t>
+    <t>El programa relocaliza de forma correcta la fila de headers, indica la max coincidencia, indica que se encuentran completos los datos, los tras data son vacios, duplicados indica que no tiene</t>
   </si>
   <si>
     <t>Desfase de Origen Vertical (Filas basura al inicio) y con header duplicados</t>
@@ -509,7 +525,7 @@
     <t>El programa debe ser capaz de reajustar el nuevo header y analizar, si encuentra algun duplicados indicar que datos estan duplicados, indicar que se encuentran completos</t>
   </si>
   <si>
-    <t>El programa esta reajusta el analisis del header y al analizarlo indica cuales son los valores que se encuentran duplicados</t>
+    <t>El programa localiza la fila de headers de forma correcta indica la coincidencia, los trash data estan como vacios, los duplicados indica que valores estan duplicados</t>
   </si>
   <si>
     <t>TC17</t>
@@ -527,7 +543,7 @@
     <t>El programa debe analizar primero las filasy saltarse esas filas encima agregadas  y columnas que no tienen datos e indicar que no tiene columnas adicionales, ni duplicados, solo debe reajustar el analisis de los headers</t>
   </si>
   <si>
-    <t>El programa deajusta el nuevo valor del encabezado e indica que datos se encuentran completos</t>
+    <t>El programa relocaliza la fila de datos, indica la coincidencia encontrada, los valores nan pos desfase vertical son encontrados y mandados a trash data, son filtrados e indica que no se encuentran duplicados</t>
   </si>
   <si>
     <t>TC18</t>
@@ -545,6 +561,9 @@
     <t>El programa debe reajustar la fila del header y analizar, indicarle al usuario que se encuentra completa, pero las columnas adicionales no seran consideradas y que no hay datos duplicados</t>
   </si>
   <si>
+    <t>El programa reloza y encuentra la fila de headers, indica la coincidencia encontrada, los comentarios o columnas encontrados adicionales se muestran como trash data, en cuanto a duplicados no se encuentra ninguno</t>
+  </si>
+  <si>
     <t>TC19</t>
   </si>
   <si>
@@ -560,7 +579,28 @@
     <t>Como los casos estan solucionados por  si solos sin errores, el programa debe ser capaz de unir todo esto e indicar si hacenfalta 1 2 o dos los encabezados aun con el defase de columna y fila y con headers intercalados duplicados algunos por lo que solo debe indicar que faltan los datos, los que se encuentran duplicados e ignirar las columnas adicionales agregadas por el usuario e ignorar las columnas que no son necesarias</t>
   </si>
   <si>
-    <t>pendig by refactor</t>
+    <t>El programa relocaliza de forma exitosa la fila de datos, se encuentran valores nan en la fila de datos y datos adicionales que son identificados como trrash data, posterior a ello identifica los faltantes y los que se encuentran duplicados de esa fila</t>
+  </si>
+  <si>
+    <t>TC20</t>
+  </si>
+  <si>
+    <t>Desfase de columna para identificar max coincidencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las filas tienen diferentes datos de header, en diferentes filas </t>
+  </si>
+  <si>
+    <t>La fila 1 puede empezar con 1 dato del header, la fila 2 con 2 datos de header, y asi de forma sucesiva, hasta la fila 8 con mayor coincidencia</t>
+  </si>
+  <si>
+    <t>El programa deje de reajustar la max coincidencia encontrada y es la que analizara</t>
+  </si>
+  <si>
+    <t>El programa recorre las filas, indica cual es la fila con mayor coincidencia y la evalua indicando que no hay duplicados o faltantes</t>
+  </si>
+  <si>
+    <t>TC21</t>
   </si>
   <si>
     <t>Inconsistencia de Case (Mayús/Minús)</t>
@@ -572,6 +612,9 @@
     <t>Falta de coincidencia ortográfica exacta en los encabezados de las columnas. Si el proceso busca "Campaign" y el archivo tiene "campaign" o "CAMPAIGN"</t>
   </si>
   <si>
+    <t>TC22</t>
+  </si>
+  <si>
     <t>Ruido por Espacios en Blanco (Strip)</t>
   </si>
   <si>
@@ -581,6 +624,9 @@
     <t>La columa A1 contiene la informacion requerida pero en esta hay espacios (ej. "date " en lugar de "date")</t>
   </si>
   <si>
+    <t>TC23</t>
+  </si>
+  <si>
     <t>Ruido por espacios e Inconsistencia de Case (Mayus/Minus) y duplicados</t>
   </si>
   <si>
@@ -590,6 +636,9 @@
     <t>Los encaezados continen espacio y discrepancia de mayus y minus ejemplo ("DATE " y "DATE" o " date" )ect  y variantes y tiene datos duplicados</t>
   </si>
   <si>
+    <t>TC24</t>
+  </si>
+  <si>
     <t>Ruido por inconsistencia de Case Mayus/Minus Duplicados y Col extras</t>
   </si>
   <si>
@@ -599,6 +648,9 @@
     <t>Lo encanezados continen espacio y discrepancia de mayus y minus ejemplo ("DATE " y "DATE" o " date" )ect  y variantes y tiene filas extras ejemplo Comentarios de juan</t>
   </si>
   <si>
+    <t>TC25</t>
+  </si>
+  <si>
     <t>Diplicados de Datos</t>
   </si>
   <si>
@@ -606,6 +658,9 @@
   </si>
   <si>
     <t>Existen datos duplicados en los encabezados es decide "date" y "date " adicionalmente el archivo tiene columas dedatos adicionales que agrego el usuario ejemplo "Comentarios de Juanito" y eliminarlas, no tomarlas en cuenta</t>
+  </si>
+  <si>
+    <t>TC26</t>
   </si>
   <si>
     <t>Evaluacion de filas extra</t>
@@ -662,7 +717,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -693,12 +748,6 @@
         <bgColor rgb="FFF1C232"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor theme="7"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -720,7 +769,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="38">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -769,16 +818,10 @@
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -793,37 +836,19 @@
     <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="6" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -832,19 +857,16 @@
     <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -860,7 +882,7 @@
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -968,6 +990,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
+<file path=xl/drawings/drawing18.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
@@ -1005,8 +1031,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I33" displayName="Tabla_1" name="Tabla_1" id="1">
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H35" displayName="Tabla_1" name="Tabla_1" id="1">
+  <tableColumns count="8">
     <tableColumn name="Case Number" id="1"/>
     <tableColumn name="Defecto a revisar" id="2"/>
     <tableColumn name="Descripcion" id="3"/>
@@ -1015,7 +1041,6 @@
     <tableColumn name="Status" id="6"/>
     <tableColumn name="Justificacion del caso" id="7"/>
     <tableColumn name="Actual Result" id="8"/>
-    <tableColumn name="Columna 1" id="9"/>
   </tableColumns>
   <tableStyleInfo name="TC Codigo-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
@@ -4697,6 +4722,149 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="C3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="18.38"/>
     <col customWidth="1" min="2" max="2" width="18.0"/>
@@ -5105,7 +5273,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -5146,694 +5314,717 @@
       <c r="H1" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="I1" s="13" t="s">
-        <v>79</v>
-      </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="14" t="s">
         <v>42</v>
       </c>
       <c r="B2" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="D2" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="E2" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="F2" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="F2" s="14" t="s">
+      <c r="G2" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="H2" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="H2" s="14" t="s">
+    </row>
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="I2" s="16"/>
-    </row>
-    <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" s="17" t="s">
+      <c r="C3" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="D3" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="D3" s="17" t="s">
+      <c r="E3" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="F3" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+    </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="19"/>
-    </row>
-    <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="B4" s="17" t="s">
+      <c r="C4" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="D4" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="E4" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="F4" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+    </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="F4" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="19"/>
-    </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="17" t="s">
+      <c r="C5" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="D5" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="E5" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="F5" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+    </row>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="F5" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="19"/>
-    </row>
-    <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="17" t="s">
+      <c r="C6" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="D6" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="E6" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="F6" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+    </row>
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="18"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+    </row>
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="F6" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="19"/>
-    </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="20"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="21"/>
-    </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="20"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
-      <c r="I8" s="21"/>
-    </row>
-    <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="22" t="s">
+      <c r="B9" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="C9" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+    </row>
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C10" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="A11" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G11" s="22"/>
+      <c r="H11" s="14" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" ht="22.5" customHeight="1">
+      <c r="A12" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G12" s="22"/>
+      <c r="H12" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="13" ht="22.5" customHeight="1">
+      <c r="A13" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13" s="22"/>
+      <c r="H13" s="14" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="G14" s="22"/>
+      <c r="H14" s="14" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>131</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>132</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15" s="25"/>
+      <c r="H15" s="23" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="16" ht="22.5" customHeight="1">
+      <c r="A16" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="F16" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G16" s="22"/>
+      <c r="H16" s="14" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="17" ht="22.5" customHeight="1">
+      <c r="A17" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G17" s="22"/>
+      <c r="H17" s="14" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="18" ht="22.5" customHeight="1">
+      <c r="A18" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G18" s="22"/>
+      <c r="H18" s="14" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="A19" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G19" s="22"/>
+      <c r="H19" s="14" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G20" s="22"/>
+      <c r="H20" s="14" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G21" s="26"/>
+      <c r="H21" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G22" s="26"/>
+      <c r="H22" s="14" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G23" s="22"/>
+      <c r="H23" s="14" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G24" s="22"/>
+      <c r="H24" s="14" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="F25" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G25" s="22"/>
+      <c r="H25" s="14" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="27"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="19"/>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="27"/>
+      <c r="B27" s="27"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="19"/>
+      <c r="H27" s="19"/>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="C28" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D28" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="23"/>
-      <c r="H9" s="23"/>
-      <c r="I9" s="24"/>
-    </row>
-    <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="25" t="s">
-        <v>56</v>
-      </c>
-      <c r="B10" s="26" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="26" t="s">
-        <v>107</v>
-      </c>
-      <c r="D10" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="E10" s="26" t="s">
-        <v>109</v>
-      </c>
-      <c r="F10" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="I10" s="16"/>
-    </row>
-    <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" s="26" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" s="26" t="s">
-        <v>112</v>
-      </c>
-      <c r="D11" s="26" t="s">
-        <v>113</v>
-      </c>
-      <c r="E11" s="26" t="s">
-        <v>114</v>
-      </c>
-      <c r="F11" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="G11" s="27"/>
-      <c r="H11" s="26" t="s">
-        <v>115</v>
-      </c>
-      <c r="I11" s="16"/>
-    </row>
-    <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="25" t="s">
-        <v>53</v>
-      </c>
-      <c r="B12" s="26" t="s">
-        <v>116</v>
-      </c>
-      <c r="C12" s="26" t="s">
-        <v>117</v>
-      </c>
-      <c r="D12" s="26" t="s">
-        <v>118</v>
-      </c>
-      <c r="E12" s="26" t="s">
-        <v>119</v>
-      </c>
-      <c r="F12" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="G12" s="27"/>
-      <c r="H12" s="26" t="s">
-        <v>120</v>
-      </c>
-      <c r="I12" s="16"/>
-    </row>
-    <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="26" t="s">
-        <v>121</v>
-      </c>
-      <c r="C13" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="D13" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="E13" s="26" t="s">
-        <v>124</v>
-      </c>
-      <c r="F13" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="G13" s="27"/>
-      <c r="H13" s="26" t="s">
-        <v>125</v>
-      </c>
-      <c r="I13" s="28" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="26" t="s">
-        <v>127</v>
-      </c>
-      <c r="C14" s="26" t="s">
-        <v>128</v>
-      </c>
-      <c r="D14" s="26" t="s">
-        <v>129</v>
-      </c>
-      <c r="E14" s="26" t="s">
-        <v>130</v>
-      </c>
-      <c r="F14" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="G14" s="27"/>
-      <c r="H14" s="26" t="s">
-        <v>131</v>
-      </c>
-      <c r="I14" s="16"/>
-    </row>
-    <row r="15" ht="22.5" customHeight="1">
-      <c r="A15" s="29" t="s">
-        <v>66</v>
-      </c>
-      <c r="B15" s="30" t="s">
-        <v>132</v>
-      </c>
-      <c r="C15" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="D15" s="30" t="s">
-        <v>134</v>
-      </c>
-      <c r="E15" s="31" t="s">
-        <v>135</v>
-      </c>
-      <c r="F15" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="G15" s="32"/>
-      <c r="H15" s="30" t="s">
-        <v>136</v>
-      </c>
-      <c r="I15" s="21"/>
-    </row>
-    <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="B16" s="26" t="s">
-        <v>137</v>
-      </c>
-      <c r="C16" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="D16" s="26" t="s">
-        <v>139</v>
-      </c>
-      <c r="E16" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="F16" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="G16" s="27"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="21"/>
-    </row>
-    <row r="17" ht="22.5" customHeight="1">
-      <c r="A17" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="B17" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="C17" s="26" t="s">
-        <v>142</v>
-      </c>
-      <c r="D17" s="26" t="s">
-        <v>143</v>
-      </c>
-      <c r="E17" s="26" t="s">
-        <v>144</v>
-      </c>
-      <c r="F17" s="26" t="s">
-        <v>145</v>
-      </c>
-      <c r="G17" s="33"/>
-      <c r="H17" s="33"/>
-      <c r="I17" s="21"/>
-    </row>
-    <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="B18" s="26" t="s">
-        <v>146</v>
-      </c>
-      <c r="C18" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="D18" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="E18" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="F18" s="26" t="s">
-        <v>145</v>
-      </c>
-      <c r="G18" s="27"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="21"/>
-    </row>
-    <row r="19" ht="22.5" customHeight="1">
-      <c r="A19" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B19" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="C19" s="26" t="s">
-        <v>151</v>
-      </c>
-      <c r="D19" s="26" t="s">
-        <v>152</v>
-      </c>
-      <c r="E19" s="26" t="s">
-        <v>153</v>
-      </c>
-      <c r="F19" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="G19" s="27"/>
-      <c r="H19" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="I19" s="16"/>
-    </row>
-    <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" s="26" t="s">
-        <v>156</v>
-      </c>
-      <c r="C20" s="26" t="s">
-        <v>157</v>
-      </c>
-      <c r="D20" s="26" t="s">
-        <v>158</v>
-      </c>
-      <c r="E20" s="26" t="s">
-        <v>159</v>
-      </c>
-      <c r="F20" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="G20" s="34"/>
-      <c r="H20" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="I20" s="16"/>
-    </row>
-    <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="25" t="s">
-        <v>161</v>
-      </c>
-      <c r="B21" s="26" t="s">
-        <v>162</v>
-      </c>
-      <c r="C21" s="26" t="s">
-        <v>163</v>
-      </c>
-      <c r="D21" s="26" t="s">
-        <v>164</v>
-      </c>
-      <c r="E21" s="26" t="s">
-        <v>165</v>
-      </c>
-      <c r="F21" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="G21" s="34"/>
-      <c r="H21" s="26" t="s">
-        <v>166</v>
-      </c>
-      <c r="I21" s="16"/>
-    </row>
-    <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="B22" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="C22" s="26" t="s">
-        <v>169</v>
-      </c>
-      <c r="D22" s="26" t="s">
-        <v>170</v>
-      </c>
-      <c r="E22" s="26" t="s">
-        <v>171</v>
-      </c>
-      <c r="F22" s="26"/>
-      <c r="G22" s="33"/>
-      <c r="H22" s="33"/>
-      <c r="I22" s="21"/>
-    </row>
-    <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="26" t="s">
-        <v>172</v>
-      </c>
-      <c r="B23" s="26" t="s">
-        <v>173</v>
-      </c>
-      <c r="C23" s="26" t="s">
-        <v>174</v>
-      </c>
-      <c r="D23" s="26" t="s">
-        <v>175</v>
-      </c>
-      <c r="E23" s="26" t="s">
-        <v>176</v>
-      </c>
-      <c r="F23" s="26" t="s">
-        <v>177</v>
-      </c>
-      <c r="G23" s="33"/>
-      <c r="H23" s="33"/>
-      <c r="I23" s="21"/>
-    </row>
-    <row r="24" ht="22.5" customHeight="1">
-      <c r="A24" s="35"/>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="21"/>
-    </row>
-    <row r="25" ht="22.5" customHeight="1">
-      <c r="A25" s="35"/>
-      <c r="B25" s="35"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="35"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
-    </row>
-    <row r="26" ht="22.5" customHeight="1">
-      <c r="A26" s="22" t="s">
-        <v>104</v>
-      </c>
-      <c r="B26" s="22" t="s">
-        <v>105</v>
-      </c>
-      <c r="C26" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="D26" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="E26" s="36"/>
-      <c r="F26" s="36"/>
-      <c r="G26" s="36"/>
-      <c r="H26" s="36"/>
-      <c r="I26" s="37"/>
-    </row>
-    <row r="27" ht="22.5" customHeight="1">
-      <c r="A27" s="38" t="s">
-        <v>70</v>
-      </c>
-      <c r="B27" s="26" t="s">
-        <v>178</v>
-      </c>
-      <c r="C27" s="26" t="s">
-        <v>179</v>
-      </c>
-      <c r="D27" s="26" t="s">
-        <v>180</v>
-      </c>
-      <c r="E27" s="39"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="40"/>
-      <c r="H27" s="40"/>
-      <c r="I27" s="41"/>
-    </row>
-    <row r="28" ht="22.5" customHeight="1">
-      <c r="A28" s="38" t="s">
-        <v>64</v>
-      </c>
-      <c r="B28" s="26" t="s">
-        <v>181</v>
-      </c>
-      <c r="C28" s="26" t="s">
-        <v>182</v>
-      </c>
-      <c r="D28" s="26" t="s">
-        <v>183</v>
-      </c>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="40"/>
-      <c r="H28" s="40"/>
-      <c r="I28" s="41"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28"/>
     </row>
     <row r="29" ht="22.5" customHeight="1">
-      <c r="A29" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="B29" s="26" t="s">
-        <v>184</v>
-      </c>
-      <c r="C29" s="26" t="s">
-        <v>185</v>
-      </c>
-      <c r="D29" s="26" t="s">
-        <v>186</v>
-      </c>
-      <c r="E29" s="39"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="40"/>
-      <c r="H29" s="40"/>
-      <c r="I29" s="41"/>
+      <c r="A29" s="29" t="s">
+        <v>190</v>
+      </c>
+      <c r="B29" s="30" t="s">
+        <v>191</v>
+      </c>
+      <c r="C29" s="30" t="s">
+        <v>192</v>
+      </c>
+      <c r="D29" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
     </row>
     <row r="30" ht="22.5" customHeight="1">
-      <c r="A30" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="B30" s="26" t="s">
-        <v>187</v>
-      </c>
-      <c r="C30" s="26" t="s">
-        <v>188</v>
-      </c>
-      <c r="D30" s="26" t="s">
-        <v>189</v>
-      </c>
-      <c r="E30" s="39"/>
-      <c r="F30" s="39"/>
-      <c r="G30" s="40"/>
-      <c r="H30" s="40"/>
-      <c r="I30" s="41"/>
+      <c r="A30" s="29" t="s">
+        <v>194</v>
+      </c>
+      <c r="B30" s="30" t="s">
+        <v>195</v>
+      </c>
+      <c r="C30" s="30" t="s">
+        <v>196</v>
+      </c>
+      <c r="D30" s="30" t="s">
+        <v>197</v>
+      </c>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
     </row>
     <row r="31" ht="22.5" customHeight="1">
-      <c r="A31" s="42" t="s">
-        <v>167</v>
-      </c>
-      <c r="B31" s="43" t="s">
-        <v>190</v>
-      </c>
-      <c r="C31" s="43" t="s">
-        <v>191</v>
-      </c>
-      <c r="D31" s="26" t="s">
-        <v>192</v>
-      </c>
-      <c r="E31" s="44"/>
-      <c r="F31" s="44"/>
-      <c r="G31" s="45"/>
-      <c r="H31" s="45"/>
-      <c r="I31" s="46"/>
+      <c r="A31" s="29" t="s">
+        <v>198</v>
+      </c>
+      <c r="B31" s="30" t="s">
+        <v>199</v>
+      </c>
+      <c r="C31" s="30" t="s">
+        <v>200</v>
+      </c>
+      <c r="D31" s="30" t="s">
+        <v>201</v>
+      </c>
+      <c r="E31" s="31"/>
+      <c r="F31" s="31"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
     </row>
     <row r="32" ht="22.5" customHeight="1">
-      <c r="A32" s="43" t="s">
-        <v>172</v>
-      </c>
-      <c r="B32" s="43" t="s">
-        <v>193</v>
-      </c>
-      <c r="C32" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="D32" s="26" t="s">
-        <v>195</v>
-      </c>
-      <c r="E32" s="44"/>
-      <c r="F32" s="44"/>
-      <c r="G32" s="45"/>
-      <c r="H32" s="45"/>
-      <c r="I32" s="46"/>
+      <c r="A32" s="29" t="s">
+        <v>202</v>
+      </c>
+      <c r="B32" s="30" t="s">
+        <v>203</v>
+      </c>
+      <c r="C32" s="30" t="s">
+        <v>204</v>
+      </c>
+      <c r="D32" s="30" t="s">
+        <v>205</v>
+      </c>
+      <c r="E32" s="31"/>
+      <c r="F32" s="31"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
     </row>
     <row r="33" ht="22.5" customHeight="1">
-      <c r="A33" s="35"/>
-      <c r="B33" s="35"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
+      <c r="A33" s="33" t="s">
+        <v>206</v>
+      </c>
+      <c r="B33" s="34" t="s">
+        <v>207</v>
+      </c>
+      <c r="C33" s="34" t="s">
+        <v>208</v>
+      </c>
+      <c r="D33" s="30" t="s">
+        <v>209</v>
+      </c>
       <c r="E33" s="35"/>
       <c r="F33" s="35"/>
-      <c r="G33" s="41"/>
-      <c r="H33" s="41"/>
-      <c r="I33" s="41"/>
-    </row>
-    <row r="35">
-      <c r="C35" s="7"/>
-    </row>
-    <row r="36">
-      <c r="B36" s="7"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="B42" s="7" t="s">
-        <v>197</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="D42" s="7" t="s">
-        <v>199</v>
+      <c r="G33" s="36"/>
+      <c r="H33" s="36"/>
+    </row>
+    <row r="34" ht="22.5" customHeight="1">
+      <c r="A34" s="34" t="s">
+        <v>210</v>
+      </c>
+      <c r="B34" s="34" t="s">
+        <v>211</v>
+      </c>
+      <c r="C34" s="34" t="s">
+        <v>212</v>
+      </c>
+      <c r="D34" s="30" t="s">
+        <v>213</v>
+      </c>
+      <c r="E34" s="35"/>
+      <c r="F34" s="35"/>
+      <c r="G34" s="36"/>
+      <c r="H34" s="36"/>
+    </row>
+    <row r="35" ht="22.5" customHeight="1">
+      <c r="A35" s="27"/>
+      <c r="B35" s="27"/>
+      <c r="C35" s="27"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="37"/>
+      <c r="H35" s="37"/>
+    </row>
+    <row r="37">
+      <c r="C37" s="7"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="7"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: TC21 tested (read_header normalization works); pseudocode for header_filter normalization pending
</commit_message>
<xml_diff>
--- a/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
+++ b/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
@@ -19,8 +19,9 @@
     <sheet state="visible" name="TC18" sheetId="14" r:id="rId18"/>
     <sheet state="visible" name="TC19" sheetId="15" r:id="rId19"/>
     <sheet state="visible" name="TC20" sheetId="16" r:id="rId20"/>
-    <sheet state="visible" name="Estructura logica" sheetId="17" r:id="rId21"/>
-    <sheet state="visible" name="TC Codigo" sheetId="18" r:id="rId22"/>
+    <sheet state="visible" name="TC21" sheetId="17" r:id="rId21"/>
+    <sheet state="visible" name="Estructura logica" sheetId="18" r:id="rId22"/>
+    <sheet state="visible" name="TC Codigo" sheetId="19" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1021" uniqueCount="226">
   <si>
     <t>date</t>
   </si>
@@ -112,6 +113,30 @@
   </si>
   <si>
     <t>Test</t>
+  </si>
+  <si>
+    <t>DATE</t>
+  </si>
+  <si>
+    <t>CAMPAIGN</t>
+  </si>
+  <si>
+    <t>CHANNEL</t>
+  </si>
+  <si>
+    <t>IMPRESSIONS</t>
+  </si>
+  <si>
+    <t>TOTAL_CLICK</t>
+  </si>
+  <si>
+    <t>SPEND</t>
+  </si>
+  <si>
+    <t>VIDEO_VIEWS</t>
+  </si>
+  <si>
+    <t>CONVERSION</t>
   </si>
   <si>
     <t>Path ok</t>
@@ -769,7 +794,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -795,6 +820,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="1" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
@@ -991,6 +1019,10 @@
 </file>
 
 <file path=xl/drawings/drawing18.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing19.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -4865,6 +4897,44 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="18.38"/>
     <col customWidth="1" min="2" max="2" width="18.0"/>
@@ -4876,396 +4946,396 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>37</v>
+        <v>44</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>40</v>
+        <v>47</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>42</v>
+        <v>49</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>44</v>
+        <v>51</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>46</v>
+        <v>53</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>51</v>
+        <v>44</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>52</v>
+        <v>44</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>53</v>
+        <v>44</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>56</v>
+        <v>63</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>57</v>
+        <v>44</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="F24" s="10" t="s">
-        <v>62</v>
+        <v>44</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="F25" s="10" t="s">
-        <v>64</v>
+        <v>71</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="F26" s="10" t="s">
-        <v>66</v>
+        <v>73</v>
+      </c>
+      <c r="F26" s="11" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F27" s="10" t="s">
-        <v>68</v>
+        <v>75</v>
+      </c>
+      <c r="F27" s="11" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="F28" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="F29" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
+      </c>
+      <c r="F29" s="11" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -5273,7 +5343,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -5290,722 +5360,722 @@
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="B1" s="11" t="s">
+      <c r="A1" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+    </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+    </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+    </row>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+    </row>
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="19"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="19"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+    </row>
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+    </row>
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="A11" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" s="23"/>
+      <c r="H11" s="15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="12" ht="22.5" customHeight="1">
+      <c r="A12" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12" s="23"/>
+      <c r="H12" s="15" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="13" ht="22.5" customHeight="1">
+      <c r="A13" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" s="23"/>
+      <c r="H13" s="15" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="G14" s="23"/>
+      <c r="H14" s="15" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>140</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>141</v>
+      </c>
+      <c r="E15" s="24" t="s">
+        <v>142</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" s="26"/>
+      <c r="H15" s="24" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="16" ht="22.5" customHeight="1">
+      <c r="A16" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G16" s="23"/>
+      <c r="H16" s="15" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="17" ht="22.5" customHeight="1">
+      <c r="A17" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="F17" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G17" s="23"/>
+      <c r="H17" s="15" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="18" ht="22.5" customHeight="1">
+      <c r="A18" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="F18" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G18" s="23"/>
+      <c r="H18" s="15" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="A19" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G19" s="23"/>
+      <c r="H19" s="15" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="C1" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="F1" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="G1" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="H1" s="13" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="D2" s="14" t="s">
+      <c r="B20" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="F20" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G20" s="23"/>
+      <c r="H20" s="15" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G21" s="27"/>
+      <c r="H21" s="15" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="F22" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G22" s="27"/>
+      <c r="H22" s="15" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="F23" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G23" s="23"/>
+      <c r="H23" s="15" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="E24" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="F24" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G24" s="23"/>
+      <c r="H24" s="15" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="15" t="s">
+        <v>192</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="F25" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G25" s="23"/>
+      <c r="H25" s="15" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="28"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="20"/>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="28"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="20"/>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="B28" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="C28" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="D28" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="G2" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="H2" s="14" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-    </row>
-    <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
-    </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>95</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-    </row>
-    <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-    </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="18"/>
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-    </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="18"/>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="19"/>
-    </row>
-    <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="20" t="s">
-        <v>103</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>104</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="21"/>
-    </row>
-    <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G11" s="22"/>
-      <c r="H11" s="14" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="D12" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="F12" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G12" s="22"/>
-      <c r="H12" s="14" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="C13" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="D13" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G13" s="22"/>
-      <c r="H13" s="14" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="G14" s="22"/>
-      <c r="H14" s="14" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="15" ht="22.5" customHeight="1">
-      <c r="A15" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="B15" s="24" t="s">
-        <v>131</v>
-      </c>
-      <c r="C15" s="24" t="s">
-        <v>132</v>
-      </c>
-      <c r="D15" s="24" t="s">
-        <v>133</v>
-      </c>
-      <c r="E15" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="F15" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G15" s="25"/>
-      <c r="H15" s="23" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>139</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G16" s="22"/>
-      <c r="H16" s="14" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="17" ht="22.5" customHeight="1">
-      <c r="A17" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>141</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="D17" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="F17" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G17" s="22"/>
-      <c r="H17" s="14" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="D18" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="F18" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G18" s="22"/>
-      <c r="H18" s="14" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="19" ht="22.5" customHeight="1">
-      <c r="A19" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>151</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="D19" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="F19" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G19" s="22"/>
-      <c r="H19" s="14" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="E20" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G20" s="22"/>
-      <c r="H20" s="14" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>163</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="F21" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G21" s="26"/>
-      <c r="H21" s="14" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="14" t="s">
-        <v>166</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>169</v>
-      </c>
-      <c r="E22" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="F22" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G22" s="26"/>
-      <c r="H22" s="14" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="E23" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="F23" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G23" s="22"/>
-      <c r="H23" s="14" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="24" ht="22.5" customHeight="1">
-      <c r="A24" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="D24" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="E24" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="F24" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G24" s="22"/>
-      <c r="H24" s="14" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="25" ht="22.5" customHeight="1">
-      <c r="A25" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="D25" s="14" t="s">
-        <v>187</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="F25" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="G25" s="22"/>
-      <c r="H25" s="14" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="26" ht="22.5" customHeight="1">
-      <c r="A26" s="27"/>
-      <c r="B26" s="27"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="19"/>
-    </row>
-    <row r="27" ht="22.5" customHeight="1">
-      <c r="A27" s="27"/>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19"/>
-    </row>
-    <row r="28" ht="22.5" customHeight="1">
-      <c r="A28" s="20" t="s">
-        <v>103</v>
-      </c>
-      <c r="B28" s="20" t="s">
-        <v>104</v>
-      </c>
-      <c r="C28" s="20" t="s">
-        <v>73</v>
-      </c>
-      <c r="D28" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="29"/>
     </row>
     <row r="29" ht="22.5" customHeight="1">
-      <c r="A29" s="29" t="s">
-        <v>190</v>
-      </c>
-      <c r="B29" s="30" t="s">
-        <v>191</v>
-      </c>
-      <c r="C29" s="30" t="s">
-        <v>192</v>
-      </c>
-      <c r="D29" s="30" t="s">
-        <v>193</v>
-      </c>
-      <c r="E29" s="31"/>
-      <c r="F29" s="31"/>
-      <c r="G29" s="32"/>
-      <c r="H29" s="32"/>
+      <c r="A29" s="30" t="s">
+        <v>198</v>
+      </c>
+      <c r="B29" s="31" t="s">
+        <v>199</v>
+      </c>
+      <c r="C29" s="31" t="s">
+        <v>200</v>
+      </c>
+      <c r="D29" s="31" t="s">
+        <v>201</v>
+      </c>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="33"/>
+      <c r="H29" s="33"/>
     </row>
     <row r="30" ht="22.5" customHeight="1">
-      <c r="A30" s="29" t="s">
-        <v>194</v>
-      </c>
-      <c r="B30" s="30" t="s">
-        <v>195</v>
-      </c>
-      <c r="C30" s="30" t="s">
-        <v>196</v>
-      </c>
-      <c r="D30" s="30" t="s">
-        <v>197</v>
-      </c>
-      <c r="E30" s="31"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
+      <c r="A30" s="30" t="s">
+        <v>202</v>
+      </c>
+      <c r="B30" s="31" t="s">
+        <v>203</v>
+      </c>
+      <c r="C30" s="31" t="s">
+        <v>204</v>
+      </c>
+      <c r="D30" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="33"/>
     </row>
     <row r="31" ht="22.5" customHeight="1">
-      <c r="A31" s="29" t="s">
-        <v>198</v>
-      </c>
-      <c r="B31" s="30" t="s">
-        <v>199</v>
-      </c>
-      <c r="C31" s="30" t="s">
-        <v>200</v>
-      </c>
-      <c r="D31" s="30" t="s">
-        <v>201</v>
-      </c>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="32"/>
+      <c r="A31" s="30" t="s">
+        <v>206</v>
+      </c>
+      <c r="B31" s="31" t="s">
+        <v>207</v>
+      </c>
+      <c r="C31" s="31" t="s">
+        <v>208</v>
+      </c>
+      <c r="D31" s="31" t="s">
+        <v>209</v>
+      </c>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="33"/>
     </row>
     <row r="32" ht="22.5" customHeight="1">
-      <c r="A32" s="29" t="s">
-        <v>202</v>
-      </c>
-      <c r="B32" s="30" t="s">
-        <v>203</v>
-      </c>
-      <c r="C32" s="30" t="s">
-        <v>204</v>
-      </c>
-      <c r="D32" s="30" t="s">
-        <v>205</v>
-      </c>
-      <c r="E32" s="31"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="32"/>
-      <c r="H32" s="32"/>
+      <c r="A32" s="30" t="s">
+        <v>210</v>
+      </c>
+      <c r="B32" s="31" t="s">
+        <v>211</v>
+      </c>
+      <c r="C32" s="31" t="s">
+        <v>212</v>
+      </c>
+      <c r="D32" s="31" t="s">
+        <v>213</v>
+      </c>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="33"/>
     </row>
     <row r="33" ht="22.5" customHeight="1">
-      <c r="A33" s="33" t="s">
-        <v>206</v>
-      </c>
-      <c r="B33" s="34" t="s">
-        <v>207</v>
-      </c>
-      <c r="C33" s="34" t="s">
-        <v>208</v>
-      </c>
-      <c r="D33" s="30" t="s">
-        <v>209</v>
-      </c>
-      <c r="E33" s="35"/>
-      <c r="F33" s="35"/>
-      <c r="G33" s="36"/>
-      <c r="H33" s="36"/>
+      <c r="A33" s="34" t="s">
+        <v>214</v>
+      </c>
+      <c r="B33" s="35" t="s">
+        <v>215</v>
+      </c>
+      <c r="C33" s="35" t="s">
+        <v>216</v>
+      </c>
+      <c r="D33" s="31" t="s">
+        <v>217</v>
+      </c>
+      <c r="E33" s="36"/>
+      <c r="F33" s="36"/>
+      <c r="G33" s="37"/>
+      <c r="H33" s="37"/>
     </row>
     <row r="34" ht="22.5" customHeight="1">
-      <c r="A34" s="34" t="s">
-        <v>210</v>
-      </c>
-      <c r="B34" s="34" t="s">
-        <v>211</v>
-      </c>
-      <c r="C34" s="34" t="s">
-        <v>212</v>
-      </c>
-      <c r="D34" s="30" t="s">
-        <v>213</v>
-      </c>
-      <c r="E34" s="35"/>
-      <c r="F34" s="35"/>
-      <c r="G34" s="36"/>
-      <c r="H34" s="36"/>
+      <c r="A34" s="35" t="s">
+        <v>218</v>
+      </c>
+      <c r="B34" s="35" t="s">
+        <v>219</v>
+      </c>
+      <c r="C34" s="35" t="s">
+        <v>220</v>
+      </c>
+      <c r="D34" s="31" t="s">
+        <v>221</v>
+      </c>
+      <c r="E34" s="36"/>
+      <c r="F34" s="36"/>
+      <c r="G34" s="37"/>
+      <c r="H34" s="37"/>
     </row>
     <row r="35" ht="22.5" customHeight="1">
-      <c r="A35" s="27"/>
-      <c r="B35" s="27"/>
-      <c r="C35" s="27"/>
-      <c r="D35" s="27"/>
-      <c r="E35" s="27"/>
-      <c r="F35" s="27"/>
-      <c r="G35" s="37"/>
-      <c r="H35" s="37"/>
+      <c r="A35" s="28"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="28"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
     </row>
     <row r="37">
       <c r="C37" s="7"/>
@@ -6015,16 +6085,16 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: update TC21 test case and results in hojatest
</commit_message>
<xml_diff>
--- a/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
+++ b/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
@@ -20,8 +20,14 @@
     <sheet state="visible" name="TC19" sheetId="15" r:id="rId19"/>
     <sheet state="visible" name="TC20" sheetId="16" r:id="rId20"/>
     <sheet state="visible" name="TC21" sheetId="17" r:id="rId21"/>
-    <sheet state="visible" name="Estructura logica" sheetId="18" r:id="rId22"/>
-    <sheet state="visible" name="TC Codigo" sheetId="19" r:id="rId23"/>
+    <sheet state="visible" name="TC22" sheetId="18" r:id="rId22"/>
+    <sheet state="visible" name="TC23" sheetId="19" r:id="rId23"/>
+    <sheet state="visible" name="TC24" sheetId="20" r:id="rId24"/>
+    <sheet state="visible" name="TC25" sheetId="21" r:id="rId25"/>
+    <sheet state="visible" name="TC26" sheetId="22" r:id="rId26"/>
+    <sheet state="visible" name="Estructura logica" sheetId="23" r:id="rId27"/>
+    <sheet state="visible" name="Hoja 42" sheetId="24" r:id="rId28"/>
+    <sheet state="visible" name="TC Codigo" sheetId="25" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -29,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1021" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1119" uniqueCount="270">
   <si>
     <t>date</t>
   </si>
@@ -115,28 +121,91 @@
     <t>Test</t>
   </si>
   <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Capaign</t>
+  </si>
+  <si>
+    <t>Channel</t>
+  </si>
+  <si>
+    <t>Impressions</t>
+  </si>
+  <si>
+    <t>Total_Click</t>
+  </si>
+  <si>
+    <t>Spend</t>
+  </si>
+  <si>
+    <t>Video_views</t>
+  </si>
+  <si>
+    <t>Conversion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     impressions </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  channel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  video_views</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  total_click </t>
+  </si>
+  <si>
+    <t xml:space="preserve">     conversion</t>
+  </si>
+  <si>
     <t>DATE</t>
   </si>
   <si>
-    <t>CAMPAIGN</t>
+    <t>Total_click</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        DATE</t>
   </si>
   <si>
     <t>CHANNEL</t>
   </si>
   <si>
-    <t>IMPRESSIONS</t>
-  </si>
-  <si>
-    <t>TOTAL_CLICK</t>
-  </si>
-  <si>
-    <t>SPEND</t>
-  </si>
-  <si>
-    <t>VIDEO_VIEWS</t>
-  </si>
-  <si>
-    <t>CONVERSION</t>
+    <t xml:space="preserve">   CAMPAIGN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Impressions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Total_Click</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Video_Views</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Conversion     </t>
+  </si>
+  <si>
+    <t>Extra</t>
+  </si>
+  <si>
+    <t>Comentarios de Vana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   impressions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Date1</t>
+  </si>
+  <si>
+    <t>Campaign</t>
+  </si>
+  <si>
+    <t>Capaign2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Impression   </t>
   </si>
   <si>
     <t>Path ok</t>
@@ -268,6 +337,60 @@
     <t>TC14</t>
   </si>
   <si>
+    <t>Completitud</t>
+  </si>
+  <si>
+    <t>Duplicados</t>
+  </si>
+  <si>
+    <t>Filas extra</t>
+  </si>
+  <si>
+    <t>Resultado</t>
+  </si>
+  <si>
+    <t>Mensaje</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>Pasa</t>
+  </si>
+  <si>
+    <t>Exitoso, estan completos, archivo limpio</t>
+  </si>
+  <si>
+    <t>si</t>
+  </si>
+  <si>
+    <t>no pasa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se encuentran completos, pero hay datos duplicados, debe revisar esos duplicados </t>
+  </si>
+  <si>
+    <t>Los datos se encuentran completos las columnas adicionales seran ignoradas</t>
+  </si>
+  <si>
+    <t>No pasa</t>
+  </si>
+  <si>
+    <t>Se encuentran completos, pero tambien hay duplicados que deben ser revisados antes de insertar datos y se encuentran columnas extras que seran ignoradas</t>
+  </si>
+  <si>
+    <t>Los headers estan incompletos y hay filas extras, se debe revisar el archivo</t>
+  </si>
+  <si>
+    <t>Headers incompletos indicas los duplicados y los faltantes para que se revise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicas que headers estan incompletos, y mostrar que hay filas extras que seran ignoradas </t>
+  </si>
+  <si>
+    <t>Indicar que no se encuentran completos, hay valores duplicados que revisar antes de insertarse e indicar que columnas extra seran ignoradas</t>
+  </si>
+  <si>
     <t>Case Number</t>
   </si>
   <si>
@@ -637,6 +760,15 @@
     <t>Falta de coincidencia ortográfica exacta en los encabezados de las columnas. Si el proceso busca "Campaign" y el archivo tiene "campaign" o "CAMPAIGN"</t>
   </si>
   <si>
+    <t>El programa debe transformas los strings para validar que los headers realmente coinciden e indicar el porcentaje de coincidencia, tambien indicar si con estas mayuscuculas o datos transformados se encuentra algun duplicado</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t>El programa leyo el header y fue capas de ajustar la coincidencia con los datos transformados de mayusculas a minusculas</t>
+  </si>
+  <si>
     <t>TC22</t>
   </si>
   <si>
@@ -649,6 +781,9 @@
     <t>La columa A1 contiene la informacion requerida pero en esta hay espacios (ej. "date " en lugar de "date")</t>
   </si>
   <si>
+    <t>El programa debe ser capaz de idetnificar y eliminar los espacios agregados en el header en caso de tenerlo como se menciona en las notas "date " es lo mismo que "date" y debe indicar si se encuentran duplicados</t>
+  </si>
+  <si>
     <t>TC23</t>
   </si>
   <si>
@@ -661,40 +796,43 @@
     <t>Los encaezados continen espacio y discrepancia de mayus y minus ejemplo ("DATE " y "DATE" o " date" )ect  y variantes y tiene datos duplicados</t>
   </si>
   <si>
+    <t>El programa debe transforma los strings debido en letra minusculas y quitando espacios agregados para poder calcular la coincidencia real de los headers e indicar que se encuentran duplicados en caso de estarlos</t>
+  </si>
+  <si>
     <t>TC24</t>
   </si>
   <si>
-    <t>Ruido por inconsistencia de Case Mayus/Minus Duplicados y Col extras</t>
+    <t>Ruido por inconsistencia de Case Mayus/Minus con espacios en blanco (strips) Duplicados y Col extras</t>
   </si>
   <si>
     <t>Lo encanezados continen espacio y discrepancia de mayus y minus ejemplo ("DATE " y "DATE" o " date" )ect  y variantes y tiene columnas extras</t>
   </si>
   <si>
-    <t>Lo encanezados continen espacio y discrepancia de mayus y minus ejemplo ("DATE " y "DATE" o " date" )ect  y variantes y tiene filas extras ejemplo Comentarios de juan</t>
+    <t>Lo encabezados contienen espacio y discrepancia de mayus y minus ejemplo ("DATE " y "DATE" o " date" )ect  y variantes y tiene filas extras ejemplo Comentarios de juan, se encuentran completos los datos unicamente tiene variable de mayus y minus</t>
+  </si>
+  <si>
+    <t>El programa debe ajustar todo a minusculas y string y poder analizar el contenido de la fila para indicar la coincidencia encontrada, omitir los que son comentarios extras e indicar los duplicados</t>
   </si>
   <si>
     <t>TC25</t>
   </si>
   <si>
-    <t>Diplicados de Datos</t>
-  </si>
-  <si>
-    <t>El archivo tiene duplicado y tiene filas extras de informacion</t>
-  </si>
-  <si>
-    <t>Existen datos duplicados en los encabezados es decide "date" y "date " adicionalmente el archivo tiene columas dedatos adicionales que agrego el usuario ejemplo "Comentarios de Juanito" y eliminarlas, no tomarlas en cuenta</t>
-  </si>
-  <si>
-    <t>TC26</t>
-  </si>
-  <si>
-    <t>Evaluacion de filas extra</t>
-  </si>
-  <si>
-    <t>El archivo contiene filas de informacion adicional</t>
-  </si>
-  <si>
-    <t>Existen filas de informacion adicional agregadas por el usuario ejemplo "Comentarios de juan" las cuales no deben serconsideras, la informacion se encuentra completa</t>
+    <t>Evaluacion de alfanumericos con duplicados</t>
+  </si>
+  <si>
+    <t>El archivo vontiene headers como date1 date2 campaign 1es decir alfanumericos</t>
+  </si>
+  <si>
+    <t>El programa contiene informacion adicional en algunos headers como date1, date2, date 3, se encuentran completos pero con duplicados</t>
+  </si>
+  <si>
+    <t>Los datos deben ser transformados y evaluados como string sin espacios, para poder poder la fila de mayor coincidencia e indicar los que se encuentran duplicados</t>
+  </si>
+  <si>
+    <t>TC27</t>
+  </si>
+  <si>
+    <t>Mosntercase</t>
   </si>
   <si>
     <t xml:space="preserve">TC_X — </t>
@@ -895,10 +1033,10 @@
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1027,6 +1165,30 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing20.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing21.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing22.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing23.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing24.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing25.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -4935,6 +5097,603 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="5">
+        <v>5168.0</v>
+      </c>
+      <c r="E1" s="5">
+        <v>134.0</v>
+      </c>
+      <c r="F1" s="5">
+        <v>258.0</v>
+      </c>
+      <c r="G1" s="4">
+        <v>362.0</v>
+      </c>
+      <c r="H1" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="5">
+        <v>2314.0</v>
+      </c>
+      <c r="E2" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="F2" s="5">
+        <v>162.0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>46.0</v>
+      </c>
+      <c r="H2" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5">
+        <v>3496.0</v>
+      </c>
+      <c r="E3" s="5">
+        <v>92.0</v>
+      </c>
+      <c r="F3" s="5">
+        <v>61.0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="H3" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1790.0</v>
+      </c>
+      <c r="E4" s="5">
+        <v>87.0</v>
+      </c>
+      <c r="F4" s="5">
+        <v>370.0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>54.0</v>
+      </c>
+      <c r="H4" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="5">
+        <v>9764.0</v>
+      </c>
+      <c r="E5" s="5">
+        <v>53.0</v>
+      </c>
+      <c r="F5" s="5">
+        <v>118.0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>293.0</v>
+      </c>
+      <c r="H5" s="6">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="5">
+        <v>2912.0</v>
+      </c>
+      <c r="E6" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="F6" s="5">
+        <v>187.0</v>
+      </c>
+      <c r="G6" s="4">
+        <v>204.0</v>
+      </c>
+      <c r="H6" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="5">
+        <v>4736.0</v>
+      </c>
+      <c r="E7" s="5">
+        <v>123.0</v>
+      </c>
+      <c r="F7" s="5">
+        <v>198.0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>237.0</v>
+      </c>
+      <c r="H7" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="5">
+        <v>7311.0</v>
+      </c>
+      <c r="E8" s="5">
+        <v>149.0</v>
+      </c>
+      <c r="F8" s="5">
+        <v>230.0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>219.0</v>
+      </c>
+      <c r="H8" s="6">
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="5">
+        <v>4679.0</v>
+      </c>
+      <c r="E9" s="5">
+        <v>22.0</v>
+      </c>
+      <c r="F9" s="5">
+        <v>281.0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>94.0</v>
+      </c>
+      <c r="H9" s="6">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="5">
+        <v>4957.0</v>
+      </c>
+      <c r="E10" s="5">
+        <v>93.0</v>
+      </c>
+      <c r="F10" s="5">
+        <v>276.0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>397.0</v>
+      </c>
+      <c r="H10" s="6">
+        <v>5.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="5">
+        <v>2924.0</v>
+      </c>
+      <c r="E11" s="5">
+        <v>131.0</v>
+      </c>
+      <c r="F11" s="5">
+        <v>58.0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>175.0</v>
+      </c>
+      <c r="H11" s="6">
+        <v>7.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="5">
+        <v>7200.0</v>
+      </c>
+      <c r="E12" s="5">
+        <v>96.0</v>
+      </c>
+      <c r="F12" s="5">
+        <v>315.0</v>
+      </c>
+      <c r="G12" s="6">
+        <v>288.0</v>
+      </c>
+      <c r="H12" s="6">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="5">
+        <v>2177.0</v>
+      </c>
+      <c r="E13" s="5">
+        <v>23.0</v>
+      </c>
+      <c r="F13" s="5">
+        <v>262.0</v>
+      </c>
+      <c r="G13" s="6">
+        <v>131.0</v>
+      </c>
+      <c r="H13" s="6">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <v>45658.0</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="5">
+        <v>4367.0</v>
+      </c>
+      <c r="E14" s="5">
+        <v>126.0</v>
+      </c>
+      <c r="F14" s="5">
+        <v>161.0</v>
+      </c>
+      <c r="G14" s="6">
+        <v>262.0</v>
+      </c>
+      <c r="H14" s="6">
+        <v>6.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="3">
+      <c r="B3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="18.38"/>
     <col customWidth="1" min="2" max="2" width="18.0"/>
@@ -4946,396 +5705,549 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>37</v>
+        <v>58</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>41</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>51</v>
+        <v>72</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="s">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>58</v>
+        <v>79</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>41</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>59</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>60</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>63</v>
+        <v>84</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>64</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>67</v>
+        <v>88</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>68</v>
+        <v>89</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>70</v>
+        <v>91</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>76</v>
+        <v>97</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>77</v>
+        <v>98</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>78</v>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -5343,7 +6255,18 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -5361,140 +6284,140 @@
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
       <c r="A1" s="12" t="s">
-        <v>79</v>
+        <v>118</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>82</v>
+        <v>121</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>83</v>
+        <v>122</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>84</v>
+        <v>123</v>
       </c>
       <c r="G1" s="14" t="s">
-        <v>85</v>
+        <v>124</v>
       </c>
       <c r="H1" s="14" t="s">
-        <v>86</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="15" t="s">
-        <v>50</v>
+        <v>71</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>87</v>
+        <v>126</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>88</v>
+        <v>127</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>89</v>
+        <v>128</v>
       </c>
       <c r="E2" s="16" t="s">
-        <v>90</v>
+        <v>129</v>
       </c>
       <c r="F2" s="15" t="s">
-        <v>91</v>
+        <v>130</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>92</v>
+        <v>131</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>93</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="17" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>94</v>
+        <v>133</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>95</v>
+        <v>134</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>96</v>
+        <v>135</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>97</v>
+        <v>136</v>
       </c>
       <c r="F3" s="17" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="G3" s="18"/>
       <c r="H3" s="18"/>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="17" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>99</v>
+        <v>138</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>101</v>
+        <v>140</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>102</v>
+        <v>141</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="G4" s="18"/>
       <c r="H4" s="18"/>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="17" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>103</v>
+        <v>142</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>105</v>
+        <v>144</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>106</v>
+        <v>145</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="G5" s="18"/>
       <c r="H5" s="18"/>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="17" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>107</v>
+        <v>146</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>108</v>
+        <v>147</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>109</v>
+        <v>148</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>110</v>
+        <v>149</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
@@ -5521,16 +6444,16 @@
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="21" t="s">
-        <v>111</v>
+        <v>150</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>112</v>
+        <v>151</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>82</v>
+        <v>121</v>
       </c>
       <c r="E9" s="21"/>
       <c r="F9" s="21"/>
@@ -5539,386 +6462,386 @@
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="15" t="s">
-        <v>64</v>
+        <v>85</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>113</v>
+        <v>152</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>114</v>
+        <v>153</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>115</v>
+        <v>154</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>116</v>
+        <v>155</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G10" s="15"/>
       <c r="H10" s="15" t="s">
-        <v>117</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="15" t="s">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>118</v>
+        <v>157</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>119</v>
+        <v>158</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>120</v>
+        <v>159</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>121</v>
+        <v>160</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G11" s="23"/>
       <c r="H11" s="15" t="s">
-        <v>122</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="15" t="s">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>123</v>
+        <v>162</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>124</v>
+        <v>163</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>125</v>
+        <v>164</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>126</v>
+        <v>165</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G12" s="23"/>
       <c r="H12" s="15" t="s">
-        <v>127</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="15" t="s">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>128</v>
+        <v>167</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>129</v>
+        <v>168</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>130</v>
+        <v>169</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>131</v>
+        <v>170</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G13" s="23"/>
       <c r="H13" s="15" t="s">
-        <v>132</v>
+        <v>171</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="15" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>133</v>
+        <v>172</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>134</v>
+        <v>173</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>135</v>
+        <v>174</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>136</v>
+        <v>175</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>137</v>
+        <v>176</v>
       </c>
       <c r="G14" s="23"/>
       <c r="H14" s="15" t="s">
-        <v>138</v>
+        <v>177</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="24" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="B15" s="25" t="s">
-        <v>139</v>
+        <v>178</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>140</v>
+        <v>179</v>
       </c>
       <c r="D15" s="25" t="s">
-        <v>141</v>
+        <v>180</v>
       </c>
       <c r="E15" s="24" t="s">
-        <v>142</v>
+        <v>181</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G15" s="26"/>
       <c r="H15" s="24" t="s">
-        <v>143</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="15" t="s">
-        <v>76</v>
+        <v>97</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>144</v>
+        <v>183</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>145</v>
+        <v>184</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>146</v>
+        <v>185</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>147</v>
+        <v>186</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G16" s="23"/>
       <c r="H16" s="15" t="s">
-        <v>148</v>
+        <v>187</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="15" t="s">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>149</v>
+        <v>188</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>150</v>
+        <v>189</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>151</v>
+        <v>190</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>152</v>
+        <v>191</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G17" s="23"/>
       <c r="H17" s="15" t="s">
-        <v>153</v>
+        <v>192</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="15" t="s">
-        <v>154</v>
+        <v>193</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>155</v>
+        <v>194</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>156</v>
+        <v>195</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>157</v>
+        <v>196</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G18" s="23"/>
       <c r="H18" s="15" t="s">
-        <v>158</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="15" t="s">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>159</v>
+        <v>198</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>160</v>
+        <v>199</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>161</v>
+        <v>200</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>162</v>
+        <v>201</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G19" s="23"/>
       <c r="H19" s="15" t="s">
-        <v>163</v>
+        <v>202</v>
       </c>
     </row>
     <row r="20" ht="22.5" customHeight="1">
       <c r="A20" s="15" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>164</v>
+        <v>203</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>165</v>
+        <v>204</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>166</v>
+        <v>205</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>167</v>
+        <v>206</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G20" s="23"/>
       <c r="H20" s="15" t="s">
-        <v>168</v>
+        <v>207</v>
       </c>
     </row>
     <row r="21" ht="22.5" customHeight="1">
       <c r="A21" s="15" t="s">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>169</v>
+        <v>208</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>170</v>
+        <v>209</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>171</v>
+        <v>210</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>172</v>
+        <v>211</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G21" s="27"/>
       <c r="H21" s="15" t="s">
-        <v>173</v>
+        <v>212</v>
       </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="15" t="s">
-        <v>174</v>
+        <v>213</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>175</v>
+        <v>214</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>176</v>
+        <v>215</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>177</v>
+        <v>216</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>178</v>
+        <v>217</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G22" s="27"/>
       <c r="H22" s="15" t="s">
-        <v>179</v>
+        <v>218</v>
       </c>
     </row>
     <row r="23" ht="22.5" customHeight="1">
       <c r="A23" s="15" t="s">
-        <v>180</v>
+        <v>219</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>181</v>
+        <v>220</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>182</v>
+        <v>221</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>184</v>
+        <v>223</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G23" s="23"/>
       <c r="H23" s="15" t="s">
-        <v>185</v>
+        <v>224</v>
       </c>
     </row>
     <row r="24" ht="22.5" customHeight="1">
       <c r="A24" s="15" t="s">
-        <v>186</v>
+        <v>225</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>187</v>
+        <v>226</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>188</v>
+        <v>227</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>189</v>
+        <v>228</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>190</v>
+        <v>229</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G24" s="23"/>
       <c r="H24" s="15" t="s">
-        <v>191</v>
+        <v>230</v>
       </c>
     </row>
     <row r="25" ht="22.5" customHeight="1">
       <c r="A25" s="15" t="s">
-        <v>192</v>
+        <v>231</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>193</v>
+        <v>232</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>194</v>
+        <v>233</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>195</v>
+        <v>234</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>196</v>
+        <v>235</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="G25" s="23"/>
       <c r="H25" s="15" t="s">
-        <v>197</v>
+        <v>236</v>
       </c>
     </row>
     <row r="26" ht="22.5" customHeight="1">
@@ -5943,16 +6866,16 @@
     </row>
     <row r="28" ht="22.5" customHeight="1">
       <c r="A28" s="21" t="s">
-        <v>111</v>
+        <v>150</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>112</v>
+        <v>151</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>82</v>
+        <v>121</v>
       </c>
       <c r="E28" s="29"/>
       <c r="F28" s="29"/>
@@ -5961,111 +6884,121 @@
     </row>
     <row r="29" ht="22.5" customHeight="1">
       <c r="A29" s="30" t="s">
-        <v>198</v>
+        <v>237</v>
       </c>
       <c r="B29" s="31" t="s">
-        <v>199</v>
+        <v>238</v>
       </c>
       <c r="C29" s="31" t="s">
-        <v>200</v>
+        <v>239</v>
       </c>
       <c r="D29" s="31" t="s">
-        <v>201</v>
-      </c>
-      <c r="E29" s="32"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="33"/>
-      <c r="H29" s="33"/>
+        <v>240</v>
+      </c>
+      <c r="E29" s="31" t="s">
+        <v>241</v>
+      </c>
+      <c r="F29" s="31" t="s">
+        <v>242</v>
+      </c>
+      <c r="G29" s="32"/>
+      <c r="H29" s="33" t="s">
+        <v>243</v>
+      </c>
     </row>
     <row r="30" ht="22.5" customHeight="1">
       <c r="A30" s="30" t="s">
-        <v>202</v>
+        <v>244</v>
       </c>
       <c r="B30" s="31" t="s">
-        <v>203</v>
+        <v>245</v>
       </c>
       <c r="C30" s="31" t="s">
-        <v>204</v>
+        <v>246</v>
       </c>
       <c r="D30" s="31" t="s">
-        <v>205</v>
-      </c>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="33"/>
-      <c r="H30" s="33"/>
+        <v>247</v>
+      </c>
+      <c r="E30" s="31" t="s">
+        <v>248</v>
+      </c>
+      <c r="F30" s="34"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
     </row>
     <row r="31" ht="22.5" customHeight="1">
       <c r="A31" s="30" t="s">
-        <v>206</v>
+        <v>249</v>
       </c>
       <c r="B31" s="31" t="s">
-        <v>207</v>
+        <v>250</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>208</v>
+        <v>251</v>
       </c>
       <c r="D31" s="31" t="s">
-        <v>209</v>
-      </c>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="33"/>
-      <c r="H31" s="33"/>
+        <v>252</v>
+      </c>
+      <c r="E31" s="31" t="s">
+        <v>253</v>
+      </c>
+      <c r="F31" s="34"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
     </row>
     <row r="32" ht="22.5" customHeight="1">
       <c r="A32" s="30" t="s">
-        <v>210</v>
+        <v>254</v>
       </c>
       <c r="B32" s="31" t="s">
-        <v>211</v>
+        <v>255</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>212</v>
+        <v>256</v>
       </c>
       <c r="D32" s="31" t="s">
-        <v>213</v>
-      </c>
-      <c r="E32" s="32"/>
-      <c r="F32" s="32"/>
-      <c r="G32" s="33"/>
-      <c r="H32" s="33"/>
+        <v>257</v>
+      </c>
+      <c r="E32" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="F32" s="34"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
     </row>
     <row r="33" ht="22.5" customHeight="1">
-      <c r="A33" s="34" t="s">
-        <v>214</v>
-      </c>
-      <c r="B33" s="35" t="s">
-        <v>215</v>
-      </c>
-      <c r="C33" s="35" t="s">
-        <v>216</v>
+      <c r="A33" s="35" t="s">
+        <v>259</v>
+      </c>
+      <c r="B33" s="31" t="s">
+        <v>260</v>
+      </c>
+      <c r="C33" s="31" t="s">
+        <v>261</v>
       </c>
       <c r="D33" s="31" t="s">
-        <v>217</v>
-      </c>
-      <c r="E33" s="36"/>
+        <v>262</v>
+      </c>
+      <c r="E33" s="31" t="s">
+        <v>263</v>
+      </c>
       <c r="F33" s="36"/>
       <c r="G33" s="37"/>
       <c r="H33" s="37"/>
     </row>
     <row r="34" ht="22.5" customHeight="1">
-      <c r="A34" s="35" t="s">
-        <v>218</v>
-      </c>
-      <c r="B34" s="35" t="s">
-        <v>219</v>
-      </c>
-      <c r="C34" s="35" t="s">
-        <v>220</v>
-      </c>
-      <c r="D34" s="31" t="s">
-        <v>221</v>
-      </c>
-      <c r="E34" s="36"/>
-      <c r="F34" s="36"/>
-      <c r="G34" s="37"/>
-      <c r="H34" s="37"/>
+      <c r="A34" s="19" t="s">
+        <v>264</v>
+      </c>
+      <c r="B34" s="19" t="s">
+        <v>265</v>
+      </c>
+      <c r="C34" s="28"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="28"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
     </row>
     <row r="35" ht="22.5" customHeight="1">
       <c r="A35" s="28"/>
@@ -6085,16 +7018,16 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="s">
-        <v>222</v>
+        <v>266</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>223</v>
+        <v>267</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>224</v>
+        <v>268</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>225</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -6102,382 +7035,6 @@
   <tableParts count="1">
     <tablePart r:id="rId3"/>
   </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1" s="5">
-        <v>5168.0</v>
-      </c>
-      <c r="E1" s="5">
-        <v>134.0</v>
-      </c>
-      <c r="F1" s="5">
-        <v>258.0</v>
-      </c>
-      <c r="G1" s="4">
-        <v>362.0</v>
-      </c>
-      <c r="H1" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="5">
-        <v>2314.0</v>
-      </c>
-      <c r="E2" s="5">
-        <v>26.0</v>
-      </c>
-      <c r="F2" s="5">
-        <v>162.0</v>
-      </c>
-      <c r="G2" s="4">
-        <v>46.0</v>
-      </c>
-      <c r="H2" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="5">
-        <v>3496.0</v>
-      </c>
-      <c r="E3" s="5">
-        <v>92.0</v>
-      </c>
-      <c r="F3" s="5">
-        <v>61.0</v>
-      </c>
-      <c r="G3" s="4">
-        <v>175.0</v>
-      </c>
-      <c r="H3" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="5">
-        <v>1790.0</v>
-      </c>
-      <c r="E4" s="5">
-        <v>87.0</v>
-      </c>
-      <c r="F4" s="5">
-        <v>370.0</v>
-      </c>
-      <c r="G4" s="4">
-        <v>54.0</v>
-      </c>
-      <c r="H4" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="5">
-        <v>9764.0</v>
-      </c>
-      <c r="E5" s="5">
-        <v>53.0</v>
-      </c>
-      <c r="F5" s="5">
-        <v>118.0</v>
-      </c>
-      <c r="G5" s="4">
-        <v>293.0</v>
-      </c>
-      <c r="H5" s="6">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="5">
-        <v>2912.0</v>
-      </c>
-      <c r="E6" s="5">
-        <v>26.0</v>
-      </c>
-      <c r="F6" s="5">
-        <v>187.0</v>
-      </c>
-      <c r="G6" s="4">
-        <v>204.0</v>
-      </c>
-      <c r="H6" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="5">
-        <v>4736.0</v>
-      </c>
-      <c r="E7" s="5">
-        <v>123.0</v>
-      </c>
-      <c r="F7" s="5">
-        <v>198.0</v>
-      </c>
-      <c r="G7" s="4">
-        <v>237.0</v>
-      </c>
-      <c r="H7" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="5">
-        <v>7311.0</v>
-      </c>
-      <c r="E8" s="5">
-        <v>149.0</v>
-      </c>
-      <c r="F8" s="5">
-        <v>230.0</v>
-      </c>
-      <c r="G8" s="4">
-        <v>219.0</v>
-      </c>
-      <c r="H8" s="6">
-        <v>4.0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="5">
-        <v>4679.0</v>
-      </c>
-      <c r="E9" s="5">
-        <v>22.0</v>
-      </c>
-      <c r="F9" s="5">
-        <v>281.0</v>
-      </c>
-      <c r="G9" s="4">
-        <v>94.0</v>
-      </c>
-      <c r="H9" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="5">
-        <v>4957.0</v>
-      </c>
-      <c r="E10" s="5">
-        <v>93.0</v>
-      </c>
-      <c r="F10" s="5">
-        <v>276.0</v>
-      </c>
-      <c r="G10" s="4">
-        <v>397.0</v>
-      </c>
-      <c r="H10" s="6">
-        <v>5.0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="5">
-        <v>2924.0</v>
-      </c>
-      <c r="E11" s="5">
-        <v>131.0</v>
-      </c>
-      <c r="F11" s="5">
-        <v>58.0</v>
-      </c>
-      <c r="G11" s="4">
-        <v>175.0</v>
-      </c>
-      <c r="H11" s="6">
-        <v>7.0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="5">
-        <v>7200.0</v>
-      </c>
-      <c r="E12" s="5">
-        <v>96.0</v>
-      </c>
-      <c r="F12" s="5">
-        <v>315.0</v>
-      </c>
-      <c r="G12" s="6">
-        <v>288.0</v>
-      </c>
-      <c r="H12" s="6">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D13" s="5">
-        <v>2177.0</v>
-      </c>
-      <c r="E13" s="5">
-        <v>23.0</v>
-      </c>
-      <c r="F13" s="5">
-        <v>262.0</v>
-      </c>
-      <c r="G13" s="6">
-        <v>131.0</v>
-      </c>
-      <c r="H13" s="6">
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4">
-        <v>45658.0</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" s="5">
-        <v>4367.0</v>
-      </c>
-      <c r="E14" s="5">
-        <v>126.0</v>
-      </c>
-      <c r="F14" s="5">
-        <v>161.0</v>
-      </c>
-      <c r="G14" s="6">
-        <v>262.0</v>
-      </c>
-      <c r="H14" s="6">
-        <v>6.0</v>
-      </c>
-    </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs: document TC21-TC25 expected results and pass status
</commit_message>
<xml_diff>
--- a/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
+++ b/Portfolio/ETL-Data-Validation-Pipeline/assets/hojatest.xlsx
@@ -26,8 +26,7 @@
     <sheet state="visible" name="TC25" sheetId="21" r:id="rId25"/>
     <sheet state="visible" name="TC26" sheetId="22" r:id="rId26"/>
     <sheet state="visible" name="Estructura logica" sheetId="23" r:id="rId27"/>
-    <sheet state="visible" name="Hoja 42" sheetId="24" r:id="rId28"/>
-    <sheet state="visible" name="TC Codigo" sheetId="25" r:id="rId29"/>
+    <sheet state="visible" name="TC Codigo" sheetId="24" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1119" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1127" uniqueCount="274">
   <si>
     <t>date</t>
   </si>
@@ -784,6 +783,9 @@
     <t>El programa debe ser capaz de idetnificar y eliminar los espacios agregados en el header en caso de tenerlo como se menciona en las notas "date " es lo mismo que "date" y debe indicar si se encuentran duplicados</t>
   </si>
   <si>
+    <t xml:space="preserve">El Programa elimina los espacios antes y despues de cada palabra y ajusta a una lista limpia, indica que datos hacen falta, en este caso ninguno, indica que no hay duplicados </t>
+  </si>
+  <si>
     <t>TC23</t>
   </si>
   <si>
@@ -799,6 +801,9 @@
     <t>El programa debe transforma los strings debido en letra minusculas y quitando espacios agregados para poder calcular la coincidencia real de los headers e indicar que se encuentran duplicados en caso de estarlos</t>
   </si>
   <si>
+    <t>El programa es capaz de identificar los espacios los elimina y al transfrmar la informacion valida si se encuentra duplicada</t>
+  </si>
+  <si>
     <t>TC24</t>
   </si>
   <si>
@@ -814,6 +819,9 @@
     <t>El programa debe ajustar todo a minusculas y string y poder analizar el contenido de la fila para indicar la coincidencia encontrada, omitir los que son comentarios extras e indicar los duplicados</t>
   </si>
   <si>
+    <t>El programa identifica los espacios ideptifica duplicados, indica los que hacen falta e indica lo que se tiene como comentario extra</t>
+  </si>
+  <si>
     <t>TC25</t>
   </si>
   <si>
@@ -827,6 +835,9 @@
   </si>
   <si>
     <t>Los datos deben ser transformados y evaluados como string sin espacios, para poder poder la fila de mayor coincidencia e indicar los que se encuentran duplicados</t>
+  </si>
+  <si>
+    <t>El programa transforma los datos a string y valida que esos alfanumericos no coinciden por lo que los agrega como datos innecesarios, indica los que se encuentran duplicados y faltantes</t>
   </si>
   <si>
     <t>TC27</t>
@@ -932,7 +943,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="34">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1023,28 +1034,13 @@
     <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1185,10 +1181,6 @@
 </file>
 
 <file path=xl/drawings/drawing24.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing25.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -6261,17 +6253,6 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <sheetData/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="2" max="2" width="23.5"/>
     <col customWidth="1" min="3" max="3" width="32.5"/>
@@ -6883,122 +6864,138 @@
       <c r="H28" s="29"/>
     </row>
     <row r="29" ht="22.5" customHeight="1">
-      <c r="A29" s="30" t="s">
+      <c r="A29" s="15" t="s">
         <v>237</v>
       </c>
-      <c r="B29" s="31" t="s">
+      <c r="B29" s="15" t="s">
         <v>238</v>
       </c>
-      <c r="C29" s="31" t="s">
+      <c r="C29" s="15" t="s">
         <v>239</v>
       </c>
-      <c r="D29" s="31" t="s">
+      <c r="D29" s="15" t="s">
         <v>240</v>
       </c>
-      <c r="E29" s="31" t="s">
+      <c r="E29" s="15" t="s">
         <v>241</v>
       </c>
-      <c r="F29" s="31" t="s">
+      <c r="F29" s="15" t="s">
         <v>242</v>
       </c>
-      <c r="G29" s="32"/>
-      <c r="H29" s="33" t="s">
+      <c r="G29" s="30"/>
+      <c r="H29" s="15" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="30" ht="22.5" customHeight="1">
-      <c r="A30" s="30" t="s">
+      <c r="A30" s="15" t="s">
         <v>244</v>
       </c>
-      <c r="B30" s="31" t="s">
+      <c r="B30" s="15" t="s">
         <v>245</v>
       </c>
-      <c r="C30" s="31" t="s">
+      <c r="C30" s="15" t="s">
         <v>246</v>
       </c>
-      <c r="D30" s="31" t="s">
+      <c r="D30" s="15" t="s">
         <v>247</v>
       </c>
-      <c r="E30" s="31" t="s">
+      <c r="E30" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="F30" s="34"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
+      <c r="F30" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="G30" s="30"/>
+      <c r="H30" s="15" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="31" ht="22.5" customHeight="1">
-      <c r="A31" s="30" t="s">
-        <v>249</v>
-      </c>
-      <c r="B31" s="31" t="s">
+      <c r="A31" s="15" t="s">
         <v>250</v>
       </c>
-      <c r="C31" s="31" t="s">
+      <c r="B31" s="15" t="s">
         <v>251</v>
       </c>
-      <c r="D31" s="31" t="s">
+      <c r="C31" s="15" t="s">
         <v>252</v>
       </c>
-      <c r="E31" s="31" t="s">
+      <c r="D31" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="F31" s="34"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="32"/>
+      <c r="E31" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="F31" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="G31" s="30"/>
+      <c r="H31" s="15" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="32" ht="22.5" customHeight="1">
-      <c r="A32" s="30" t="s">
-        <v>254</v>
-      </c>
-      <c r="B32" s="31" t="s">
-        <v>255</v>
-      </c>
-      <c r="C32" s="31" t="s">
+      <c r="A32" s="15" t="s">
         <v>256</v>
       </c>
-      <c r="D32" s="31" t="s">
+      <c r="B32" s="15" t="s">
         <v>257</v>
       </c>
-      <c r="E32" s="31" t="s">
+      <c r="C32" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="F32" s="34"/>
-      <c r="G32" s="32"/>
-      <c r="H32" s="32"/>
+      <c r="D32" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="E32" s="15" t="s">
+        <v>260</v>
+      </c>
+      <c r="F32" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="G32" s="30"/>
+      <c r="H32" s="15" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="33" ht="22.5" customHeight="1">
-      <c r="A33" s="35" t="s">
-        <v>259</v>
-      </c>
-      <c r="B33" s="31" t="s">
-        <v>260</v>
-      </c>
-      <c r="C33" s="31" t="s">
-        <v>261</v>
-      </c>
-      <c r="D33" s="31" t="s">
+      <c r="A33" s="31" t="s">
         <v>262</v>
       </c>
-      <c r="E33" s="31" t="s">
+      <c r="B33" s="15" t="s">
         <v>263</v>
       </c>
-      <c r="F33" s="36"/>
-      <c r="G33" s="37"/>
-      <c r="H33" s="37"/>
+      <c r="C33" s="15" t="s">
+        <v>264</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>265</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>266</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="G33" s="32"/>
+      <c r="H33" s="31" t="s">
+        <v>267</v>
+      </c>
     </row>
     <row r="34" ht="22.5" customHeight="1">
       <c r="A34" s="19" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C34" s="28"/>
       <c r="D34" s="28"/>
       <c r="E34" s="28"/>
       <c r="F34" s="28"/>
-      <c r="G34" s="38"/>
-      <c r="H34" s="38"/>
+      <c r="G34" s="33"/>
+      <c r="H34" s="33"/>
     </row>
     <row r="35" ht="22.5" customHeight="1">
       <c r="A35" s="28"/>
@@ -7007,8 +7004,8 @@
       <c r="D35" s="28"/>
       <c r="E35" s="28"/>
       <c r="F35" s="28"/>
-      <c r="G35" s="38"/>
-      <c r="H35" s="38"/>
+      <c r="G35" s="33"/>
+      <c r="H35" s="33"/>
     </row>
     <row r="37">
       <c r="C37" s="7"/>
@@ -7018,16 +7015,16 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>